<commit_message>
feat: migrate to dynamic multi-language support driven by master.xlsx
- Refactored `update_inventory_data.py` to support dynamic languages (row 1) and category labels (row 2).
- Maintained fallback support for missing translations to gracefully fail over to the primary language.
- Migrated item structure to `{"labels": {"l1": "English", "l2": "Spanish"}}` format.
- Refactored `server.py` and `app.js` endpoints and UI components to consume dynamic data format.
- Replaced hardcoded English/Spanish toggle in the frontend (`index.html`) with a dynamic `<select>` based language dropdown.
- Updated `admin.js` to render the correct translated categories/items depending on language arrays.
</commit_message>
<xml_diff>
--- a/item master/Master.xlsx
+++ b/item master/Master.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alcohol (🍺)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fountain BIB (🧃)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beverages (🥤)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleaning (🧹)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dairy (🧀)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Disposables (🥡)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frozen &amp; Refrigerated (❄️)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dry Grocery (🌾)" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meats (🥩)" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produce (🥦)" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prepared (🍲)" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Smallwares (🍴)" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Alcohol (🍺)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fountain BIB (🧃)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Beverages (🥤)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cleaning (🧹)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Dairy (🧀)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Disposables (🥡)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Frozen &amp; Refrigerated (❄️)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Dry Grocery (🌾)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Meats (🥩)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Produce (🥦)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Prepared (🍲)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Smallwares (🍴)" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -57,11 +57,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,428 +424,448 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>l1: English</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>l2: Español</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>@category: Alcohol</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@category: Alcohol</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Blue Moon 6pk.</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Blue Moon 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Bud Light 6pk</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Bud Light 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Budweiser 6pk.</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Budweiser 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Coors Light 6pk.</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Coors Light 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Corona 6pk</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Corona 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Fat Tire Ale 6pk.</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Fat Tire Ale 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Heineken 6pk.</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Heineken 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Heineken Zero 6pk.</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Heineken Zero 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>IPA DNR 6pk.</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>IPA DNR 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>IPA F5 6pk</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>IPA F5 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>IPA Native Amber</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>IPA Native Amber</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Michelob Ultra 6pk.</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Michelob Ultra 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Michelob Ultra Zero 6pk.</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Michelob Ultra Zero 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Miller Lite 6pk.</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Miller Lite 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Modelo 6pk.</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Modelo 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Modelo Negra 6pk</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Modelo Negra 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Peroni 6pk.</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Peroni 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Sam Adams Lager</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Sam Adams Lager</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Shiner Bock 6pk.</t>
         </is>
       </c>
-      <c r="B19" s="1" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Shiner Bock 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Shock Top 6pk.</t>
         </is>
       </c>
-      <c r="B20" s="1" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Shock Top 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Stella Artois 6pk</t>
         </is>
       </c>
-      <c r="B21" s="1" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>Stella Artois 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Truly Cherry</t>
         </is>
       </c>
-      <c r="B22" s="1" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Truly cereza</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Truly Strawberry Lime</t>
         </is>
       </c>
-      <c r="B23" s="1" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Truly fresa-limón</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>XX Chelada 6pk.</t>
         </is>
       </c>
-      <c r="B24" s="1" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>XX Chelada 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>XX Lager 6pk.</t>
         </is>
       </c>
-      <c r="B25" s="1" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>XX Lager 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>XX Lager Dark 6pk.</t>
         </is>
       </c>
-      <c r="B26" s="1" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>XX Lager Dark 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Yuengling Flight 6pk</t>
         </is>
       </c>
-      <c r="B27" s="1" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>Yuengling Flight 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>Yuengling Lager 6pk</t>
         </is>
       </c>
-      <c r="B28" s="1" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>Yuengling Lager 6 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Apothic Red</t>
         </is>
       </c>
-      <c r="B29" s="1" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>Apothic Red</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Bread &amp; Butter Pinot Noir</t>
         </is>
       </c>
-      <c r="B30" s="1" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>Bread &amp; Butter Pinot Noir</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Gabbiano Chianti</t>
         </is>
       </c>
-      <c r="B31" s="1" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>Gabbiano Chianti</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Gallo .187 Cabernet Sauvignon 4pk.</t>
         </is>
       </c>
-      <c r="B32" s="1" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>Gallo .187 Cabernet Sauvignon 4 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Josh Cabernet Sauvignon</t>
         </is>
       </c>
-      <c r="B33" s="1" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Josh Cabernet Sauvignon</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Sutter Home .187 Sauvignon Blanc 4pk.</t>
         </is>
       </c>
-      <c r="B34" s="1" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>Sutter Home .187 Sauvignon Blanc 4 paquetes</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>Yellowtail Pinot Noir</t>
         </is>
       </c>
-      <c r="B35" s="1" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>Yellowtail Pinot Noir</t>
         </is>
@@ -865,212 +882,232 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>l1: English</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>l2: Español</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>@category: Produce</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@category: Productos Frescos</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Basil Fresh (each)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Albahaca fresca (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Bell Peppers (Yellow, Red,Orange) 6 pk (each)</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Pimientos morrones (amarillo, rojo, naranja) paquete de 6 (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Bell Peppers Choppers (case)</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Pimientos morrones picados (caja)</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Broccoli Florets (fresh) (case)</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Floretes de brócoli (fresco) (caja)</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Broccoli Florets (frozen) (case)</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Floretes de brócoli (congelado) (caja)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Celery 1cs</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Apio 1 caja</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Cucumber English 2 pk (each)</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Pepino inglés paquete de 2 (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Lettuce Romaine (case)</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Lechuga romana (caja)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Mushroom Medium (case)</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Champiñón mediano (caja)</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Onion Red (case)</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Cebolla roja (caja)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Onion Yellow (case)</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Cebolla amarilla (caja)</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Potato Idaho 70 ct./50 lb. (case)</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Papa Idaho 70 ct./50 lb. (caja)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Spinach Fresh (each)</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Espinaca fresca (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Tomato Cherry (case)</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Tomate cherry (caja)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Tomato Cherry Constellation (each)</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Tomate cherry Constellation (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Tomato Roma (each)</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Tomate Roma (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Tomato Slicer (case)</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Tomate para rebanar (caja)</t>
         </is>
@@ -1087,236 +1124,256 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>l1: English</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>l2: Español</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>@category: Prepared</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@category: Prepared</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Bacon Bits (qt) (each)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Trocitos de tocino (cuarto) (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Bell Pepper Chopped (qt.) (each)</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Pimiento morrón picado (cuarto) (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Boneless Bites (prepared 8 ea.)</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Boneless preparados (8 pzas.)</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Chicken Breast Cooked (4 oz.) (each)</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Pechuga de pollo cocida (4 oz.) (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Chicken Parmesan (prepared) ea.</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Pollo parmesano (preparado) unidad</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Chicken Tenders (prepared 3 ea.)</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Tiras de pollo (preparadas, 3 pzas.)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Dough Par Bake 18" (each)</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Masa prehorneada 18" (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Fettucine Alfredo (prepared) ea.</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Fettuccine Alfredo (preparado) unidad</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Italian Sausage Cooked (lb.) (each)</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Salchicha italiana cocida (lb.) (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Marinara (gal.) (each)</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Marinara (galón) (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Meatballs (ea)</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Albóndigas (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Mushroom Sliced (qt) (each)</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Champiñón rebanado (cuarto) (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Onion Diced (qt.) (each)</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Cebolla en cubos (cuarto) (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Onion Sliced (qt.) (each)</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Cebolla rebanada (cuarto) (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Pizza Sauce (gal.) (each)</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Salsa para pizza (galón) (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Spaghetti w/meatballs (prepared) ea.</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Espagueti con albóndigas (preparado) unidad</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Stromboli (prepared) ea.</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Stromboli (preparado) unidad</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Tomatos Diced (qt.) (each)</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Tomates en cubos (cuarto) (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Tomatos Sliced (qt.) (each)</t>
         </is>
       </c>
-      <c r="B19" s="1" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Tomates rebanados (cuarto) (unidad)</t>
         </is>
@@ -1333,20 +1390,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>l1: English</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>l2: Español</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>@category: Smallwares</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@category: Smallwares</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Cheese shakers</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Agitadores para queso</t>
         </is>
@@ -1363,104 +1440,124 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>l1: English</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>l2: Español</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>@category: Fountain BIB</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@category: Fountain BIB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>BIB Coca-Cola</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>BIB Coca-Cola</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>BIB Coke Zero</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>BIB Coke Zero</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>BIB Diet Coke</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>BIB Diet Coke</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>BIB Diet Dr. Pepper</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>BIB Diet Dr. Pepper</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>BIB Dr.Pepper</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>BIB Dr Pepper</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>BIB Lemonade</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>BIB limonada</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>BIB Root Beer</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>BIB root beer</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>BIB Sprite</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>BIB Sprite</t>
         </is>
@@ -1477,308 +1574,328 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>l1: English</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>l2: Español</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>@category: Beverages</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@category: Beverages</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Btl Gold Peak Tea Unsweet</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Botella de té Gold Peak sin azúcar</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Btl Henry Winehard Root Beer</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Botella Henry Winehard root beer</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Btl Henry Winehard Vanilla Cream</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Botella Henry Winehard vanilla cream</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Btl Jarritos Asst Flavors cs.</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Botella Jarritos sabores surtidos (caja)</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Btl Mexican Coca-Cola cs</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Botella Coca-Cola mexicana (caja)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Btl Mexican Sprite cs</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Botella Sprite mexicano (caja)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Btl Pellegrino Ciao Lime</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Botella Pellegrino Ciao lima</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Btl Pellegrino Ciao Orange</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Botella Pellegrino Ciao naranja</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Btl Pellegrino Mineral Water</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Botella de agua mineral Pellegrino</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Btl Topo-Chico Lime</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Botella Topo-Chico lima</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Btl Topo-Chico Original</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Botella Topo-Chico original</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Btl Water</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Botella de agua</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Can A&amp;W Root Beer</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Lata A&amp;W root beer</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Can Coca-Cola</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Lata de Coca-Cola</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Can Diet Coke</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Lata de Diet Coke</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Can Diet Dr Pepper</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Lata de Diet Dr Pepper</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Can Dr Pepper</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Lata de Dr Pepper</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Can Grape Crush</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Lata de Crush de uva</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Can Mountain Dew</t>
         </is>
       </c>
-      <c r="B19" s="1" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Lata de Mountain Dew</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Can Okolo-Homa Cream Soda</t>
         </is>
       </c>
-      <c r="B20" s="1" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Lata Okolo-Homa cream soda</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Can Okolo-Homa Root Beer</t>
         </is>
       </c>
-      <c r="B21" s="1" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>Lata Okolo-Homa root beer</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Can Orange Fanta</t>
         </is>
       </c>
-      <c r="B22" s="1" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Lata de Fanta naranja</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Can Pepsi</t>
         </is>
       </c>
-      <c r="B23" s="1" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Lata de Pepsi</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Can Sprite</t>
         </is>
       </c>
-      <c r="B24" s="1" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Lata de Sprite</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Tea automatic brew 32/3.5oz.</t>
         </is>
       </c>
-      <c r="B25" s="1" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Té para preparación automática 32/3.5 oz.</t>
         </is>
@@ -1795,104 +1912,124 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>l1: English</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>l2: Español</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>@category: Cleaning</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@category: Cleaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Bleach</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Cloro</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Dish Detergent (dawn)</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Detergente para platos (Dawn)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Floor cleaner (fabuloso purple)</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Limpiador de pisos (Fabuloso morado)</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Scrubber Stainless Steel 12/1 ct.</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Fibra de acero inoxidable 12/1 ct.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Dining Room Sanitizer</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Sanitizante para comedor</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Stainless Steel cleaner</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Limpiador para acero inoxidable</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Magic Eraser</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Borrador mágico</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Window cleaner</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Limpiavidrios</t>
         </is>
@@ -1909,224 +2046,244 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>l1: English</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>l2: Español</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>@category: Dairy</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@category: Lácteos</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>American Cheese Sliced White pkg.</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Queso americano blanco en rebanadas, paquete</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>American Cheese Sliced Yellow pkg.</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Queso americano amarillo en rebanadas, paquete</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Butter European 36/1lb.</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Mantequilla europea 36/1 lb.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Butter Unsalted 36/1lb.</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Mantequilla sin sal 36/1 lb.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Buttermilk 1cs.</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Suero de leche 1 caja</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Cream Cheese 10/3lb.</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Queso crema 10/3 lb.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Eggs 15 doz.</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Huevos 15 docenas</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Heavy Cream cs.</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Crema espesa (caja)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Mozzarella BelGioioso Fresh 2/1lb.</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Mozzarella fresca BelGioioso 2/1 lb.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Mozzarella Loaf 8/6lb.</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Mozzarella tipo loaf 8/6 lb.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Mozzarella Shredded 5lb.</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Mozzarella rallada 5 lb.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Parmesan Grated 5lb.</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Parmesano rallado 5 lb.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Parmesan Shredded 5lb.</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Parmesano deshebrado 5 lb.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Provolone sliced pkg.</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Provolone en rebanadas, paquete</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Ricotta Cheese 6/3lb.</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Queso ricotta 6/3 lb.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Sour Cream 4/5lb.</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Crema agria 4/5 lb.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Sour Cream packets</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Sobres de crema agria</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Cheddar Cheese Shredded 5lb.</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Queso cheddar rallado 5 lb.</t>
         </is>
@@ -2143,608 +2300,628 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>l1: English</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>l2: Español</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>@category: Disposables</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@category: Disposables</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>08" Ultra Lunch Paper Plate</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Plato de papel Ultra Lunch de 8"</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>10" Ultra Lunch Paper Plate</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Plato de papel Ultra Lunch de 10"</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>16 oz. Foam Cup</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Vaso de espuma de 16 oz.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>16 oz. Foam Lid</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Tapa de espuma de 16 oz.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>2 oz. Clear portion cup</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Vaso transparente para porción de 2 oz.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>2 oz. Clear Portion Lid</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Tapa transparente para porción de 2 oz.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>4 oz. Foam Portion Cup</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Vaso de espuma para porción de 4 oz.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>4 oz. Foam Portion Lid</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Tapa de espuma para porción de 4 oz.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>6x6 Clear Plastic togo</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Contenedor plástico transparente 6x6 para llevar</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>6x6 White Foam togo</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Contenedor blanco de espuma 6x6 para llevar</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>8x8 Clear togo boxes cs</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Cajas transparentes 8x8 para llevar (caja)</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>8x8 White Foam togo</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Contenedor blanco de espuma 8x8 para llevar</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>9x9 White Foam togo</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Contenedor blanco de espuma 9x9 para llevar</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Aluminum Foil Roll</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Rollo de papel aluminio</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Aluminum Foil Sheets 10.75" 1/200ct.</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Hojas de aluminio 10.75" 1/200 ct.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Aluminum Lid (FULL Pan)</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Tapa de aluminio (charola completa)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Aluminum Lid (half pan)</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Tapa de aluminio (media charola)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Aluminum Pan (FULL pan)</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Charola de aluminio (charola completa)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Aluminum Pan (half pan)</t>
         </is>
       </c>
-      <c r="B19" s="1" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Charola de aluminio (media charola)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Cutlery Fork White Heavy Duty box</t>
         </is>
       </c>
-      <c r="B20" s="1" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Caja de tenedores blancos resistentes</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Cutlery Knife White Heavy Duty box</t>
         </is>
       </c>
-      <c r="B21" s="1" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>Caja de cuchillos blancos resistentes</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Cutlery Meal Kit</t>
         </is>
       </c>
-      <c r="B22" s="1" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Kit de cubiertos</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Deli container togo 16oz.</t>
         </is>
       </c>
-      <c r="B23" s="1" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Contenedor deli para llevar de 16 oz.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Deli container togo 8oz.</t>
         </is>
       </c>
-      <c r="B24" s="1" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Contenedor deli para llevar de 8 oz.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Deli container togo lids</t>
         </is>
       </c>
-      <c r="B25" s="1" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Tapas para contenedor deli para llevar</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Dinner Knapkins</t>
         </is>
       </c>
-      <c r="B26" s="1" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>Servilletas para comida</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Film Poly 12" Wrap</t>
         </is>
       </c>
-      <c r="B27" s="1" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>Rollo de film plástico de 12"</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>Film Poly 18" Wrap</t>
         </is>
       </c>
-      <c r="B28" s="1" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>Rollo de film plástico de 18"</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Film Poly 24" Wrap</t>
         </is>
       </c>
-      <c r="B29" s="1" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>Rollo de film plástico de 24"</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Gloves Lg</t>
         </is>
       </c>
-      <c r="B30" s="1" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>Guantes grandes</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Gloves Med</t>
         </is>
       </c>
-      <c r="B31" s="1" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>Guantes medianos</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Gloves Sm</t>
         </is>
       </c>
-      <c r="B32" s="1" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>Guantes pequeños</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Menu Tissue (sgl)</t>
         </is>
       </c>
-      <c r="B33" s="1" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Papel para menú (individual)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Paper Towel (brown roll)</t>
         </is>
       </c>
-      <c r="B34" s="1" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>Toalla de papel (rollo café)</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>Paper Towels (dispenser)</t>
         </is>
       </c>
-      <c r="B35" s="1" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>Toallas de papel (dispensador)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="1" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>Paper Towels (kitchen)</t>
         </is>
       </c>
-      <c r="B36" s="1" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>Toallas de papel (cocina)</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="1" t="inlineStr">
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>Pizza Boxes 10"</t>
         </is>
       </c>
-      <c r="B37" s="1" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>Cajas para pizza de 10"</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="1" t="inlineStr">
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t>Pizza Boxes 14"</t>
         </is>
       </c>
-      <c r="B38" s="1" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>Cajas para pizza de 14"</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="1" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Pizza Boxes 18"</t>
         </is>
       </c>
-      <c r="B39" s="1" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>Cajas para pizza de 18"</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="1" t="inlineStr">
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>Portion Control Bag (sandwich size)</t>
         </is>
       </c>
-      <c r="B40" s="1" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>Bolsa de control de porción (tamaño sándwich)</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="1" t="inlineStr">
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>Register 3 1/8" Thermal Roll</t>
         </is>
       </c>
-      <c r="B41" s="1" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>Rollo térmico para caja 3 1/8"</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="1" t="inlineStr">
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>Toilet Tissue</t>
         </is>
       </c>
-      <c r="B42" s="1" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>Papel higiénico</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="1" t="inlineStr">
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>Trash Bags (kitchen size)</t>
         </is>
       </c>
-      <c r="B43" s="1" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>Bolsas de basura (tamaño cocina)</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="1" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>Trash Bags (Lg 55-65 gal)</t>
         </is>
       </c>
-      <c r="B44" s="1" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>Bolsas de basura grandes (55-65 gal.)</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="1" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>Trash Bags (Small)</t>
         </is>
       </c>
-      <c r="B45" s="1" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>Bolsas de basura pequeñas</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="1" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>T-Shirt Bag Lg.</t>
         </is>
       </c>
-      <c r="B46" s="1" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>Bolsa tipo camiseta grande</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="1" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>T-Shirt Bag Med</t>
         </is>
       </c>
-      <c r="B47" s="1" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>Bolsa tipo camiseta mediana</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="1" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>T-Shirt Bag Sm</t>
         </is>
       </c>
-      <c r="B48" s="1" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>Bolsa tipo camiseta pequeña</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="1" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>Cake Pan w/Lid</t>
         </is>
       </c>
-      <c r="B49" s="1" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>Molde para pastel con tapa</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="1" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr">
         <is>
           <t>Cake Pan rounds</t>
         </is>
       </c>
-      <c r="B50" s="1" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>Moldes redondos para pastel</t>
         </is>
@@ -2761,284 +2938,304 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>l1: English</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>l2: Español</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>@category: Frozen &amp; Refrigerated</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@category: Frozen &amp; Refrigerated</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Biscuits 1/24 cs.</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Biscuits 1/24 caja</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Cake Bundt</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Pastel bundt</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Cake Chocolate</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Pastel de chocolate</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Cake Italian Lemon Crème</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Pastel italiano de limón crème</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Cake Strawberry</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Pastel de fresa</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Cannoli Cream w/choc</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Crema de cannoli con chocolate</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Cannoli Shell Lg</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Concha de cannoli grande</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Cannoli Shell Lg (choc)</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Concha de cannoli grande (chocolate)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Cannoli Shell Sm</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Concha de cannoli pequeña</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Cannoli Shell Sm (choc)</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Concha de cannoli pequeña (chocolate)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Cheesecake NY</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Cheesecake estilo Nueva York</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Cheesecake Oreo</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Cheesecake de Oreo</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Cheesecake Turtle</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Cheesecake Turtle</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>French Fries 3/8th" Straight</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Papas fritas rectas de 3/8"</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>French Fries Crinkle Cut</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Papas fritas corte ondulado</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>French Fries Homestyle</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Papas fritas estilo casero</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>French Fries Shoestring</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Papas fritas tipo shoestring</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Hashbrown 2/10lb.</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Hashbrown 2/10 lb.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Pasta Tortellini</t>
         </is>
       </c>
-      <c r="B19" s="1" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Pasta tortellini</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Pizza Crust Cauliflower</t>
         </is>
       </c>
-      <c r="B20" s="1" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Base de pizza de coliflor</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Tater Tots</t>
         </is>
       </c>
-      <c r="B21" s="1" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>Tater tots</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Tiramisu (ea.)</t>
         </is>
       </c>
-      <c r="B22" s="1" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Tiramisú (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Tortillas Chips uncooked</t>
         </is>
       </c>
-      <c r="B23" s="1" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Totopos sin cocinar</t>
         </is>
@@ -3055,704 +3252,724 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B58"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>l1: English</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>l2: Español</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>@category: Dry Grocery</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@category: Dry Grocery</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Banana Peppers sliced 1gal.</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Chiles banana rebanados 1 gal.</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Barbecue Sauce 1 gal.</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Salsa barbecue 1 gal.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Basalmic Glaze</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Glaseado balsámico</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Black Olives Sliced #10 can/cs.</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Aceitunas negras rebanadas lata #10/caja</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Bread Baguettes</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Baguettes</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Bread Brioche Buns</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Pan brioche para hamburguesa</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Bread Crumbs Panko 25lb.</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Pan molido panko 25 lb.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Bread Hawaiian</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Pan hawaiano</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Bread Sliced Sandwich</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Pan de sándwich rebanado</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Brown Sugar 1lb.</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Azúcar morena 1 lb.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Buns Hamburger</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Pan para hamburguesa</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Buns Hot Dog</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Pan para hot dog</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Chocolate for Cannoli #10 can</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Chocolate para cannoli lata #10</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Cole Slaw Dressing 1gal.</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Aderezo para cole slaw 1 gal.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Cole Slaw mix bag</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Bolsa de mezcla para cole slaw</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Croutons 4/2.5lbs.</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Crutones 4/2.5 lb.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Dressing Caesar 1 gal</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Aderezo César 1 gal.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Dressing Italian 1 gal.</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Aderezo italiano 1 gal.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Dressing Mix Italian packet</t>
         </is>
       </c>
-      <c r="B19" s="1" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Mezcla para aderezo italiano, sobre</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Dressing Mix Ranch cs.</t>
         </is>
       </c>
-      <c r="B20" s="1" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Mezcla para aderezo ranch (caja)</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Dressing Mix Ranch packet</t>
         </is>
       </c>
-      <c r="B21" s="1" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>Mezcla para aderezo ranch, sobre</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Dressing Vinagrette 1 gal.</t>
         </is>
       </c>
-      <c r="B22" s="1" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Vinagreta 1 gal.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Everything Bagel</t>
         </is>
       </c>
-      <c r="B23" s="1" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Bagel everything</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Flour High Gluten All Trump 25lb.</t>
         </is>
       </c>
-      <c r="B24" s="1" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Harina alta en gluten All Trump 25 lb.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Flour High Gluten All Trump 50lb.</t>
         </is>
       </c>
-      <c r="B25" s="1" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Harina alta en gluten All Trump 50 lb.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Fry Oil</t>
         </is>
       </c>
-      <c r="B26" s="1" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>Aceite para freír</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Garlic Minced in water</t>
         </is>
       </c>
-      <c r="B27" s="1" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>Ajo picado en agua</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>Garlic Powder 5lb.</t>
         </is>
       </c>
-      <c r="B28" s="1" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>Ajo en polvo 5 lb.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Hot Sauce Red Hot 1 gal.</t>
         </is>
       </c>
-      <c r="B29" s="1" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>Salsa picante Red Hot 1 gal.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Jalapeno Sliced #10</t>
         </is>
       </c>
-      <c r="B30" s="1" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>Jalapeño rebanado #10</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Mayonnaise 4/1 gal.</t>
         </is>
       </c>
-      <c r="B31" s="1" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>Mayonesa 4/1 gal.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Olive Ripe Sliced #10</t>
         </is>
       </c>
-      <c r="B32" s="1" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>Aceituna madura rebanada #10</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Onion minced dried</t>
         </is>
       </c>
-      <c r="B33" s="1" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Cebolla seca picada</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Onion Powder</t>
         </is>
       </c>
-      <c r="B34" s="1" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>Cebolla en polvo</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>Oreos pkg.</t>
         </is>
       </c>
-      <c r="B35" s="1" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>Galletas Oreo, paquete</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="1" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>Packets Parmesan</t>
         </is>
       </c>
-      <c r="B36" s="1" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>Sobres de parmesano</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="1" t="inlineStr">
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>Packets Red Pepper cs.</t>
         </is>
       </c>
-      <c r="B37" s="1" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>Sobres de chile rojo (caja)</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="1" t="inlineStr">
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t>Pan Spray cs</t>
         </is>
       </c>
-      <c r="B38" s="1" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>Spray para sartén (caja)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="1" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Parsley minced dried</t>
         </is>
       </c>
-      <c r="B39" s="1" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>Perejil seco picado</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="1" t="inlineStr">
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>Pasta Fettucine 10"</t>
         </is>
       </c>
-      <c r="B40" s="1" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>Pasta fettuccine 10"</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="1" t="inlineStr">
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>Pasta Lasagna 10"</t>
         </is>
       </c>
-      <c r="B41" s="1" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>Pasta para lasaña 10"</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="1" t="inlineStr">
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>Pasta Penne Rigate</t>
         </is>
       </c>
-      <c r="B42" s="1" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>Pasta penne rigate</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="1" t="inlineStr">
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>Pasta Rotini Tri Color</t>
         </is>
       </c>
-      <c r="B43" s="1" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>Pasta rotini tricolor</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="1" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>Pasta Spaghetti 10"</t>
         </is>
       </c>
-      <c r="B44" s="1" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>Pasta espagueti 10"</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="1" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>Pepperoncini Whole 1 gal.</t>
         </is>
       </c>
-      <c r="B45" s="1" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>Pepperoncini entero 1 gal.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="1" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>Pineapple tidbits #10</t>
         </is>
       </c>
-      <c r="B46" s="1" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>Piña en trozos #10</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="1" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>Plain Bagel</t>
         </is>
       </c>
-      <c r="B47" s="1" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>Bagel natural</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="1" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>Salsa Fire Roasted #10</t>
         </is>
       </c>
-      <c r="B48" s="1" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>Salsa fire roasted #10</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="1" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>Salt 50lb.</t>
         </is>
       </c>
-      <c r="B49" s="1" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>Sal 50 lb.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="1" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr">
         <is>
           <t>Sugar 50lb.</t>
         </is>
       </c>
-      <c r="B50" s="1" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>Azúcar 50 lb.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="1" t="inlineStr">
+    <row r="53">
+      <c r="A53" t="inlineStr">
         <is>
           <t>Sugar Powdered bag</t>
         </is>
       </c>
-      <c r="B51" s="1" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>Azúcar glass, bolsa</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="1" t="inlineStr">
+    <row r="54">
+      <c r="A54" t="inlineStr">
         <is>
           <t>Texas Toast</t>
         </is>
       </c>
-      <c r="B52" s="1" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>Texas toast</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="1" t="inlineStr">
+    <row r="55">
+      <c r="A55" t="inlineStr">
         <is>
           <t>Tomato Paste cs.</t>
         </is>
       </c>
-      <c r="B53" s="1" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>Pasta de tomate (caja)</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="1" t="inlineStr">
+    <row r="56">
+      <c r="A56" t="inlineStr">
         <is>
           <t>Tomato Sauce cs.</t>
         </is>
       </c>
-      <c r="B54" s="1" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>Salsa de tomate (caja)</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="1" t="inlineStr">
+    <row r="57">
+      <c r="A57" t="inlineStr">
         <is>
           <t>Tortillas Flour 10"</t>
         </is>
       </c>
-      <c r="B55" s="1" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>Tortillas de harina 10"</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="1" t="inlineStr">
+    <row r="58">
+      <c r="A58" t="inlineStr">
         <is>
           <t>Vinegar Red 1 gal</t>
         </is>
       </c>
-      <c r="B56" s="1" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>Vinagre rojo 1 gal.</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="1" t="inlineStr">
+    <row r="59">
+      <c r="A59" t="inlineStr">
         <is>
           <t>Vinegar White 1 gal</t>
         </is>
       </c>
-      <c r="B57" s="1" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>Vinagre blanco 1 gal.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="1" t="inlineStr">
+    <row r="60">
+      <c r="A60" t="inlineStr">
         <is>
           <t>Yeast</t>
         </is>
       </c>
-      <c r="B58" s="1" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>Levadura</t>
         </is>
@@ -3769,224 +3986,244 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>l1: English</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>l2: Español</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>@category: Meats</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>@category: Carnes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Bacon Bits (case)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Tocino en trocitos (caja)</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Bacon Sliced 1cs</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Tocino rebanado 1 caja</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Brisket (each)</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Brisket (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Canadian Bacon (case)</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Tocino canadiense (caja)</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Catfish/Swai cs.</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Bagre/Swai (caja)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Chicken Breast (case)</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Pechuga de pollo (caja)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Chicken Wings (case)</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Alitas de pollo (caja)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Ground Beef 73/27 lbs</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Carne molida 73/27 lb.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Ground Beef 80/20 lbs</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Carne molida 80/20 lb.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Ground Beef 90/10 lbs</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Carne molida 90/10 lb.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Hot Dogs (each)</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Hot dogs (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Hot Links (each)</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Salchichas hot links (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Italian Sausage Rope (case)</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Salchicha italiana en tira (caja)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Pepperoni (case)</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Pepperoni (caja)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Philly Meat (case)</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Carne tipo Philly (caja)</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Polish Sausage (each)</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Salchicha polaca (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Pork Butt (each)</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Pork butt (unidad)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Shrimp 21-25 raw peeled 5/2lb. (case)</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Camarón 21-25 crudo pelado 5/2 lb. (caja)</t>
         </is>

</xml_diff>

<commit_message>
docs: update master inventory format guide and master sheet
Update the `docs/Master_Inventory_Format_Guide.md` document to describe the new row 1 `en`/`es` format alongside category translations on row 2.
Rebuilt `item master/Master.xlsx` to use the new layout using combined data from legacy `English Master.xlsx` and `Spanish Master.xlsx` files.
</commit_message>
<xml_diff>
--- a/item master/Master.xlsx
+++ b/item master/Master.xlsx
@@ -7,18 +7,19 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Alcohol (🍺)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Fountain BIB (🧃)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Beverages (🥤)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cleaning (🧹)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Dairy (🧀)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Disposables (🥡)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Frozen &amp; Refrigerated (❄️)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Dry Grocery (🌾)" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Meats (🥩)" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Produce (🥦)" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Prepared (🍲)" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Smallwares (🍴)" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="BEV-ALC" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="BEV-BIB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BEV-RTD" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CLEANING" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="DAIRY" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="DISPOSABLES" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="FROZEN.REF" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="GROCERY DRY" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MEATS" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="PRODUCE" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="PREPARED" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="SMALLWARES" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="BAKERY" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -424,450 +425,114 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>l1: English</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>l2: Español</t>
+          <t>es</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>@category: Alcohol</t>
+          <t>BEV-ALC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>@category: Alcohol</t>
+          <t>BEV-ALC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Blue Moon 6pk.</t>
+          <t>Stella Artois 6pk</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Blue Moon 6 paquetes</t>
+          <t>Stella Artois 6pk</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bud Light 6pk</t>
+          <t>Yuengling Flight 6pk</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bud Light 6 paquetes</t>
+          <t>Yuengling Flight 6pk</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Budweiser 6pk.</t>
+          <t>Bud Light 6pk</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Budweiser 6 paquetes</t>
+          <t>Bud Light 6pk</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Coors Light 6pk.</t>
+          <t>Modelo Negra 6pk</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Coors Light 6 paquetes</t>
+          <t>Modelo Negra 6pk</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Corona 6pk</t>
+          <t>F5 IPA 6pk</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Corona 6 paquetes</t>
+          <t>F5 IPA 6pk</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Fat Tire Ale 6pk.</t>
+          <t>Corona 6pk</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Fat Tire Ale 6 paquetes</t>
+          <t>Corona 6pk</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Heineken 6pk.</t>
+          <t>Modelo 6pk.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Heineken 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Heineken Zero 6pk.</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Heineken Zero 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>IPA DNR 6pk.</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>IPA DNR 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>IPA F5 6pk</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>IPA F5 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>IPA Native Amber</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>IPA Native Amber</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Michelob Ultra 6pk.</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Michelob Ultra 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Michelob Ultra Zero 6pk.</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Michelob Ultra Zero 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Miller Lite 6pk.</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Miller Lite 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
           <t>Modelo 6pk.</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Modelo 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Modelo Negra 6pk</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Modelo Negra 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Peroni 6pk.</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Peroni 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Sam Adams Lager</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Sam Adams Lager</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Shiner Bock 6pk.</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Shiner Bock 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Shock Top 6pk.</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Shock Top 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Stella Artois 6pk</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Stella Artois 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Truly Cherry</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Truly cereza</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Truly Strawberry Lime</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Truly fresa-limón</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>XX Chelada 6pk.</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>XX Chelada 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>XX Lager 6pk.</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>XX Lager 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>XX Lager Dark 6pk.</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>XX Lager Dark 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Yuengling Flight 6pk</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Yuengling Flight 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Yuengling Lager 6pk</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Yuengling Lager 6 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Apothic Red</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Apothic Red</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Bread &amp; Butter Pinot Noir</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Bread &amp; Butter Pinot Noir</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Gabbiano Chianti</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Gabbiano Chianti</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Gallo .187 Cabernet Sauvignon 4pk.</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Gallo .187 Cabernet Sauvignon 4 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Josh Cabernet Sauvignon</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Josh Cabernet Sauvignon</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Sutter Home .187 Sauvignon Blanc 4pk.</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Sutter Home .187 Sauvignon Blanc 4 paquetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Yellowtail Pinot Noir</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Yellowtail Pinot Noir</t>
         </is>
       </c>
     </row>
@@ -882,90 +547,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>l1: English</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>l2: Español</t>
+          <t>es</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>@category: Produce</t>
+          <t>PRODUCE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>@category: Productos Frescos</t>
+          <t>Productos Frescos</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Basil Fresh (each)</t>
+          <t>Basil Fresh</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Albahaca fresca (unidad)</t>
+          <t>Albahaca Fresca</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bell Peppers (Yellow, Red,Orange) 6 pk (each)</t>
+          <t>Bell Peppers (Yellow, Red,Orange) 6 pk</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pimientos morrones (amarillo, rojo, naranja) paquete de 6 (unidad)</t>
+          <t>Pimientos (Amarillo, Rojo, Naranja) 6 paq.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Bell Peppers Choppers (case)</t>
+          <t>Bell Peppers Choppers</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Pimientos morrones picados (caja)</t>
+          <t>Pimientos para Picar</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Broccoli Florets (fresh) (case)</t>
+          <t>Broccoli Florets (fresh)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Floretes de brócoli (fresco) (caja)</t>
+          <t>Flores de Brócoli (frescas)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Broccoli Florets (frozen) (case)</t>
+          <t>Broccoli Florets (frozen)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Floretes de brócoli (congelado) (caja)</t>
+          <t>Flores de Brócoli (congeladas)</t>
         </is>
       </c>
     </row>
@@ -984,132 +649,120 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cucumber English 2 pk (each)</t>
+          <t>Constellation Cherry Tomatoes</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pepino inglés paquete de 2 (unidad)</t>
+          <t>Tomates Cherry Constellation</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Lettuce Romaine (case)</t>
+          <t>Cucumber English 2 pk</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Lechuga romana (caja)</t>
+          <t>Pepino Inglés 2 paq.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mushroom Medium (case)</t>
+          <t>Lettuce Romaine</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Champiñón mediano (caja)</t>
+          <t>Lechuga Romana</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Onion Red (case)</t>
+          <t>Mushroom Medium</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cebolla roja (caja)</t>
+          <t>Champiñones Medianos</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Onion Yellow (case)</t>
+          <t>Onion Red</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cebolla amarilla (caja)</t>
+          <t>Cebolla Roja</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Potato Idaho 70 ct./50 lb. (case)</t>
+          <t>Onion Yellow</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Papa Idaho 70 ct./50 lb. (caja)</t>
+          <t>Cebolla Amarilla</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Spinach Fresh (each)</t>
+          <t>Potato Idaho 70 ct./50 lb.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Espinaca fresca (unidad)</t>
+          <t>Papas Idaho 70 ct./50 lb.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Tomato Cherry (case)</t>
+          <t>Spinach Fresh</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tomate cherry (caja)</t>
+          <t>Espinaca Fresca</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Tomato Cherry Constellation (each)</t>
+          <t>Tomato Cherry</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tomate cherry Constellation (unidad)</t>
+          <t>Tomates Cherry</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Tomato Roma (each)</t>
+          <t>Tomato Roma</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tomate Roma (unidad)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Tomato Slicer (case)</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Tomate para rebanar (caja)</t>
+          <t>Tomates Roma</t>
         </is>
       </c>
     </row>
@@ -1130,252 +783,252 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>l1: English</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>l2: Español</t>
+          <t>es</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>@category: Prepared</t>
+          <t>PREPARED</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>@category: Prepared</t>
+          <t>PREPARED</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bacon Bits (qt) (each)</t>
+          <t>Chicken Breast Cooked (4 oz.)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Trocitos de tocino (cuarto) (unidad)</t>
+          <t>Pechuga de Pollo Cocida (4 oz.)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bell Pepper Chopped (qt.) (each)</t>
+          <t>Boneless Bites (prepared 8 ea.)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pimiento morrón picado (cuarto) (unidad)</t>
+          <t>Trozos sin Hueso (preparados 8 c/u)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Boneless Bites (prepared 8 ea.)</t>
+          <t>Chicken Tenders (prepared 3 ea.)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Boneless preparados (8 pzas.)</t>
+          <t>Tiras de Pollo (preparadas 3 c/u)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Chicken Breast Cooked (4 oz.) (each)</t>
+          <t>Dough Par Bake 18"</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pechuga de pollo cocida (4 oz.) (unidad)</t>
+          <t>Masa Pre-cocida 18"</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Chicken Parmesan (prepared) ea.</t>
+          <t>Marinara (gal.)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Pollo parmesano (preparado) unidad</t>
+          <t>Salsa Marinara (gal.)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Chicken Tenders (prepared 3 ea.)</t>
+          <t>Pizza Sauce (gal.)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tiras de pollo (preparadas, 3 pzas.)</t>
+          <t>Salsa de Pizza (gal.)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Dough Par Bake 18" (each)</t>
+          <t>Italian Sausage Cooked (lb.)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Masa prehorneada 18" (unidad)</t>
+          <t>Salchicha Italiana Cocida (lb.)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Fettucine Alfredo (prepared) ea.</t>
+          <t>Onion Diced (qt.)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fettuccine Alfredo (preparado) unidad</t>
+          <t>Cebolla Cortada en Cubitos (cto.)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Italian Sausage Cooked (lb.) (each)</t>
+          <t>Onion Sliced (qt.)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Salchicha italiana cocida (lb.) (unidad)</t>
+          <t>Cebolla en Rodajas (cto.)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Marinara (gal.) (each)</t>
+          <t>Bell Pepper Chopped (qt.)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Marinara (galón) (unidad)</t>
+          <t>Pimiento Picado (cto.)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Meatballs (ea)</t>
+          <t>Mushroom Sliced (qt)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Albóndigas (unidad)</t>
+          <t>Champiñones en Rodajas (cto.)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mushroom Sliced (qt) (each)</t>
+          <t>Tomatos Sliced (qt.)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Champiñón rebanado (cuarto) (unidad)</t>
+          <t>Tomates en Rodajas (cto.)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Onion Diced (qt.) (each)</t>
+          <t>Tomatos Diced (qt.)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cebolla en cubos (cuarto) (unidad)</t>
+          <t>Tomates Cortados en Cubitos (cto.)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Onion Sliced (qt.) (each)</t>
+          <t>Bacon Bits (qt)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cebolla rebanada (cuarto) (unidad)</t>
+          <t>Trozos de Tocino (cto.)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Pizza Sauce (gal.) (each)</t>
+          <t>Stromboli (prepared) ea.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Salsa para pizza (galón) (unidad)</t>
+          <t>Stromboli (preparado) c/u</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Spaghetti w/meatballs (prepared) ea.</t>
+          <t>Meatballs (ea)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Espagueti con albóndigas (preparado) unidad</t>
+          <t>Albóndigas (c/u)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Stromboli (prepared) ea.</t>
+          <t>Fettucine Alfredo (prepared) ea.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Stromboli (preparado) unidad</t>
+          <t>Fettuccine Alfredo (preparado) c/u</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Tomatos Diced (qt.) (each)</t>
+          <t>Spaghetti w/meatballs (prepared) ea.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Tomates en cubos (cuarto) (unidad)</t>
+          <t>Espaguetis con Albóndigas (preparado) c/u</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Tomatos Sliced (qt.) (each)</t>
+          <t>Chicken Parmesan (prepared) ea.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Tomates rebanados (cuarto) (unidad)</t>
+          <t>Pollo a la Parmesana (preparado) c/u</t>
         </is>
       </c>
     </row>
@@ -1396,24 +1049,24 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>l1: English</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>l2: Español</t>
+          <t>es</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>@category: Smallwares</t>
+          <t>SMALLWARES</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>@category: Smallwares</t>
+          <t>SMALLWARES</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1078,57 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Agitadores para queso</t>
+          <t>Queseros</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BAKERY</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BAKERY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Film Poly 24" Wrap</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Envoltura de Película Plástica 24"</t>
         </is>
       </c>
     </row>
@@ -1446,24 +1149,24 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>l1: English</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>l2: Español</t>
+          <t>es</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>@category: Fountain BIB</t>
+          <t>BEV-BIB</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>@category: Fountain BIB</t>
+          <t>BEV-BIB</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1178,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BIB Coca-Cola</t>
+          <t>Caja de Jarabe Coca-Cola</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1190,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BIB Coke Zero</t>
+          <t>Caja de Jarabe Coke Zero</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1202,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BIB Diet Coke</t>
+          <t>Caja de Jarabe Diet Coke</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1214,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BIB Diet Dr. Pepper</t>
+          <t>Caja de Jarabe Diet Dr. Pepper</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1226,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BIB Dr Pepper</t>
+          <t>Caja de Jarabe Dr. Pepper</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1238,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BIB limonada</t>
+          <t>Caja de Jarabe Limonada</t>
         </is>
       </c>
     </row>
@@ -1547,7 +1250,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BIB root beer</t>
+          <t>Caja de Jarabe Cerveza de Raíz</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1262,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BIB Sprite</t>
+          <t>Caja de Jarabe Sprite</t>
         </is>
       </c>
     </row>
@@ -1574,330 +1277,78 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>l1: English</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>l2: Español</t>
+          <t>es</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>@category: Beverages</t>
+          <t>BEV-RTD</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>@category: Beverages</t>
+          <t>BEV-RTD</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Btl Gold Peak Tea Unsweet</t>
+          <t>Tea automatic brew 32/3.5oz.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Botella de té Gold Peak sin azúcar</t>
+          <t>Té preparado automático 32/3.5oz.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Btl Henry Winehard Root Beer</t>
+          <t>Jarritos Asst Flavors cs.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Botella Henry Winehard root beer</t>
+          <t>Jarritos Sabores Surtidos caja</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Btl Henry Winehard Vanilla Cream</t>
+          <t>Mexican Coca-Cola cs</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Botella Henry Winehard vanilla cream</t>
+          <t>Coca-Cola Mexicana caja</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Btl Jarritos Asst Flavors cs.</t>
+          <t>Mexican Sprite cs</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Botella Jarritos sabores surtidos (caja)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Btl Mexican Coca-Cola cs</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Botella Coca-Cola mexicana (caja)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Btl Mexican Sprite cs</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Botella Sprite mexicano (caja)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Btl Pellegrino Ciao Lime</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Botella Pellegrino Ciao lima</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Btl Pellegrino Ciao Orange</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Botella Pellegrino Ciao naranja</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Btl Pellegrino Mineral Water</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Botella de agua mineral Pellegrino</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Btl Topo-Chico Lime</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Botella Topo-Chico lima</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Btl Topo-Chico Original</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Botella Topo-Chico original</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Btl Water</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Botella de agua</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Can A&amp;W Root Beer</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Lata A&amp;W root beer</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Can Coca-Cola</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Lata de Coca-Cola</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Can Diet Coke</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Lata de Diet Coke</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Can Diet Dr Pepper</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Lata de Diet Dr Pepper</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Can Dr Pepper</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Lata de Dr Pepper</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Can Grape Crush</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Lata de Crush de uva</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Can Mountain Dew</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Lata de Mountain Dew</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Can Okolo-Homa Cream Soda</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Lata Okolo-Homa cream soda</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Can Okolo-Homa Root Beer</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Lata Okolo-Homa root beer</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Can Orange Fanta</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Lata de Fanta naranja</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Can Pepsi</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Lata de Pepsi</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Can Sprite</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Lata de Sprite</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Tea automatic brew 32/3.5oz.</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Té para preparación automática 32/3.5 oz.</t>
+          <t>Sprite Mexicano caja</t>
         </is>
       </c>
     </row>
@@ -1912,30 +1363,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>l1: English</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>l2: Español</t>
+          <t>es</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>@category: Cleaning</t>
+          <t>CLEANING</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>@category: Cleaning</t>
+          <t>CLEANING</t>
         </is>
       </c>
     </row>
@@ -1954,12 +1405,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dish Detergent (dawn)</t>
+          <t xml:space="preserve">Dish Detergent (dawn) </t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Detergente para platos (Dawn)</t>
+          <t>Detergente para Platos (Dawn)</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1422,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Limpiador de pisos (Fabuloso morado)</t>
+          <t>Limpiador de Pisos (Fabuloso morado)</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1434,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Fibra de acero inoxidable 12/1 ct.</t>
+          <t>Esponjas de Acero Inoxidable 12/1 ct.</t>
         </is>
       </c>
     </row>
@@ -1995,43 +1446,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sanitizante para comedor</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Stainless Steel cleaner</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Limpiador para acero inoxidable</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Magic Eraser</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Borrador mágico</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Window cleaner</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Limpiavidrios</t>
+          <t>Desinfectante para Comedor</t>
         </is>
       </c>
     </row>
@@ -2046,246 +1461,234 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>l1: English</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>l2: Español</t>
+          <t>es</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>@category: Dairy</t>
+          <t>DAIRY</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>@category: Lácteos</t>
+          <t>Lácteos</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>American Cheese Sliced White pkg.</t>
+          <t>Butter European 36/1lb.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Queso americano blanco en rebanadas, paquete</t>
+          <t>Mantequilla Europea 36/1lb.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>American Cheese Sliced Yellow pkg.</t>
+          <t>Butter Unsalted 36/1lb.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Queso americano amarillo en rebanadas, paquete</t>
+          <t>Mantequilla sin Sal 36/1lb.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Butter European 36/1lb.</t>
+          <t>Buttermilk 1cs.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mantequilla europea 36/1 lb.</t>
+          <t>Suero de Mantequilla 1 caja</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Butter Unsalted 36/1lb.</t>
+          <t>Cream Cheese 10/3lb.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mantequilla sin sal 36/1 lb.</t>
+          <t>Queso Crema 10/3lb.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Buttermilk 1cs.</t>
+          <t>Eggs 15 doz.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Suero de leche 1 caja</t>
+          <t>Huevos 15 docenas</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cream Cheese 10/3lb.</t>
+          <t>Heavy Cream cs.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Queso crema 10/3 lb.</t>
+          <t>Crema Espesa caja</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Eggs 15 doz.</t>
+          <t>Mozzarella BelGioioso Fresh 2/1lb.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Huevos 15 docenas</t>
+          <t>Mozzarella Fresca BelGioioso 2/1lb.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Heavy Cream cs.</t>
+          <t>Mozzarella Loaf 8/6lb.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Crema espesa (caja)</t>
+          <t>Barra de Mozzarella 8/6lb.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mozzarella BelGioioso Fresh 2/1lb.</t>
+          <t>Mozzarella Shredded 5lb.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mozzarella fresca BelGioioso 2/1 lb.</t>
+          <t>Mozzarella Rallada 5lb.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mozzarella Loaf 8/6lb.</t>
+          <t>Parmesan Grated 5lb.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mozzarella tipo loaf 8/6 lb.</t>
+          <t>Parmesano Rallado 5lb.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mozzarella Shredded 5lb.</t>
+          <t>Parmesan Shredded 5lb.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Mozzarella rallada 5 lb.</t>
+          <t>Parmesano en Hebras 5lb.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Parmesan Grated 5lb.</t>
+          <t>Ricotta Cheese 6/3lb.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Parmesano rallado 5 lb.</t>
+          <t>Queso Ricotta 6/3lb.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Parmesan Shredded 5lb.</t>
+          <t>Sour Cream 4/5lb.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Parmesano deshebrado 5 lb.</t>
+          <t>Crema Agria 4/5lb.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Provolone sliced pkg.</t>
+          <t>Sour Cream packets</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Provolone en rebanadas, paquete</t>
+          <t>Paquetes de Crema Agria</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ricotta Cheese 6/3lb.</t>
+          <t>Provolone sliced pkg.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Queso ricotta 6/3 lb.</t>
+          <t>Provolone en Rebanadas paq.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sour Cream 4/5lb.</t>
+          <t>American Cheese Sliced Yellow pkg.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Crema agria 4/5 lb.</t>
+          <t>Queso Americano Amarillo Rebanado paq.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sour Cream packets</t>
+          <t>American Cheese Sliced White pkg.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Sobres de crema agria</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Cheddar Cheese Shredded 5lb.</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Queso cheddar rallado 5 lb.</t>
+          <t>Queso Americano Blanco Rebanado paq.</t>
         </is>
       </c>
     </row>
@@ -2300,30 +1703,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>l1: English</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>l2: Español</t>
+          <t>es</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>@category: Disposables</t>
+          <t>DISPOSABLES</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>@category: Disposables</t>
+          <t>DISPOSABLES</t>
         </is>
       </c>
     </row>
@@ -2335,7 +1738,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Plato de papel Ultra Lunch de 8"</t>
+          <t>Plato de Papel Ultra 08"</t>
         </is>
       </c>
     </row>
@@ -2347,7 +1750,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Plato de papel Ultra Lunch de 10"</t>
+          <t>Plato de Papel Ultra 10"</t>
         </is>
       </c>
     </row>
@@ -2359,7 +1762,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Vaso de espuma de 16 oz.</t>
+          <t>Vaso de Espuma 16 oz.</t>
         </is>
       </c>
     </row>
@@ -2371,7 +1774,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tapa de espuma de 16 oz.</t>
+          <t>Tapa para Vaso de Espuma 16 oz.</t>
         </is>
       </c>
     </row>
@@ -2383,7 +1786,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Vaso transparente para porción de 2 oz.</t>
+          <t>Vasito Transparente para Porción 2 oz.</t>
         </is>
       </c>
     </row>
@@ -2395,7 +1798,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tapa transparente para porción de 2 oz.</t>
+          <t>Tapa Transparente para Porción 2 oz.</t>
         </is>
       </c>
     </row>
@@ -2407,7 +1810,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Vaso de espuma para porción de 4 oz.</t>
+          <t>Vasito de Espuma para Porción 4 oz.</t>
         </is>
       </c>
     </row>
@@ -2419,7 +1822,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tapa de espuma para porción de 4 oz.</t>
+          <t>Tapa de Espuma para Porción 4 oz.</t>
         </is>
       </c>
     </row>
@@ -2431,31 +1834,31 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Contenedor plástico transparente 6x6 para llevar</t>
+          <t>Envase de Plástico Transparente para Llevar 6x6</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>6x6 White Foam togo</t>
+          <t>8x8 Clear togo boxes cs</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Contenedor blanco de espuma 6x6 para llevar</t>
+          <t>Cajas Transparentes para Llevar 8x8 caja</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8x8 Clear togo boxes cs</t>
+          <t>6x6 White Foam togo</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cajas transparentes 8x8 para llevar (caja)</t>
+          <t>Envase de Espuma Blanca para Llevar 6x6</t>
         </is>
       </c>
     </row>
@@ -2467,7 +1870,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Contenedor blanco de espuma 8x8 para llevar</t>
+          <t>Envase de Espuma Blanca para Llevar 8x8</t>
         </is>
       </c>
     </row>
@@ -2479,7 +1882,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Contenedor blanco de espuma 9x9 para llevar</t>
+          <t>Envase de Espuma Blanca para Llevar 9x9</t>
         </is>
       </c>
     </row>
@@ -2491,7 +1894,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Rollo de papel aluminio</t>
+          <t>Rollo de Papel Aluminio</t>
         </is>
       </c>
     </row>
@@ -2503,19 +1906,19 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Hojas de aluminio 10.75" 1/200 ct.</t>
+          <t>Hojas de Papel Aluminio 10.75" 1/200 ct.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aluminum Lid (FULL Pan)</t>
+          <t>Aluminum Lid (full Pan)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tapa de aluminio (charola completa)</t>
+          <t>Tapa de Aluminio (Bandeja Completa)</t>
         </is>
       </c>
     </row>
@@ -2527,19 +1930,19 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Tapa de aluminio (media charola)</t>
+          <t>Tapa de Aluminio (Media Bandeja)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aluminum Pan (FULL pan)</t>
+          <t>Aluminum Pan (full pan)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Charola de aluminio (charola completa)</t>
+          <t>Bandeja de Aluminio (Completa)</t>
         </is>
       </c>
     </row>
@@ -2551,271 +1954,271 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Charola de aluminio (media charola)</t>
+          <t>Bandeja de Aluminio (Media)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Cutlery Fork White Heavy Duty box</t>
+          <t>Cutlery Meal Kit</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Caja de tenedores blancos resistentes</t>
+          <t>Kit de Cubiertos para Comida</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Cutlery Knife White Heavy Duty box</t>
+          <t>Deli container togo 16oz.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Caja de cuchillos blancos resistentes</t>
+          <t>Envase Deli para Llevar 16 oz.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Cutlery Meal Kit</t>
+          <t>Deli container togo 8oz.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Kit de cubiertos</t>
+          <t>Envase Deli para Llevar 8 oz.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Deli container togo 16oz.</t>
+          <t>Deli container togo lids</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Contenedor deli para llevar de 16 oz.</t>
+          <t>Tapas para Envases Deli para Llevar</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Deli container togo 8oz.</t>
+          <t>Film Poly 12" Wrap</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Contenedor deli para llevar de 8 oz.</t>
+          <t>Envoltura de Película Plástica 12"</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Deli container togo lids</t>
+          <t>Film Poly 18" Wrap</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tapas para contenedor deli para llevar</t>
+          <t>Envoltura de Película Plástica 18"</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Dinner Knapkins</t>
+          <t>Film Poly 24" Wrap</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Servilletas para comida</t>
+          <t>Envoltura de Película Plástica 24"</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Film Poly 12" Wrap</t>
+          <t>Fork White Heavy Duty box</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Rollo de film plástico de 12"</t>
+          <t>Tenedor Blanco de Alta Resistencia caja</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Film Poly 18" Wrap</t>
+          <t>Gloves Lg</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Rollo de film plástico de 18"</t>
+          <t>Guantes G</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Film Poly 24" Wrap</t>
+          <t>Gloves Med</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Rollo de film plástico de 24"</t>
+          <t>Guantes M</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Gloves Lg</t>
+          <t>Gloves Sm</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Guantes grandes</t>
+          <t>Guantes P</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Gloves Med</t>
+          <t>Knife White Heavy Duty box</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Guantes medianos</t>
+          <t>Cuchillo Blanco de Alta Resistencia caja</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Gloves Sm</t>
+          <t>Menu Tissue (sgl)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Guantes pequeños</t>
+          <t>Papel Seda para Menú (sgl)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Menu Tissue (sgl)</t>
+          <t>Paper Towel (brown roll)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Papel para menú (individual)</t>
+          <t>Toalla de Papel (Rollo Marrón)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Paper Towel (brown roll)</t>
+          <t>Paper Towels (dispenser)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Toalla de papel (rollo café)</t>
+          <t>Toallas de Papel (Dispensador)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Paper Towels (dispenser)</t>
+          <t>Paper Towels (kitchen)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Toallas de papel (dispensador)</t>
+          <t>Toallas de Papel (Cocina)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Paper Towels (kitchen)</t>
+          <t>Pizza Boxes 10"</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Toallas de papel (cocina)</t>
+          <t>Cajas de Pizza 10"</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Pizza Boxes 10"</t>
+          <t>Pizza Boxes 14"</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cajas para pizza de 10"</t>
+          <t>Cajas de Pizza 14"</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Pizza Boxes 14"</t>
+          <t>Pizza Boxes 18"</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Cajas para pizza de 14"</t>
+          <t>Cajas de Pizza 18"</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Pizza Boxes 18"</t>
+          <t>Portion Control Bag (sandwich size)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Cajas para pizza de 18"</t>
+          <t>Bolsa de Control de Porción (Tamaño Sándwich)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Portion Control Bag (sandwich size)</t>
+          <t>Register 3 1/8" Thermal Roll</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Bolsa de control de porción (tamaño sándwich)</t>
+          <t>Rollo Térmico para Registradora 3 1/8"</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Register 3 1/8" Thermal Roll</t>
+          <t>Register paper 3 1/8" Thermal</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Rollo térmico para caja 3 1/8"</t>
+          <t>Papel Térmico para Registradora 3 1/8"</t>
         </is>
       </c>
     </row>
@@ -2827,7 +2230,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Papel higiénico</t>
+          <t>Papel Higiénico</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2242,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Bolsas de basura (tamaño cocina)</t>
+          <t>Bolsas de Basura (Tamaño Cocina)</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2254,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Bolsas de basura grandes (55-65 gal.)</t>
+          <t>Bolsas de Basura (Grandes 55-65 gal)</t>
         </is>
       </c>
     </row>
@@ -2863,67 +2266,43 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Bolsas de basura pequeñas</t>
+          <t>Bolsas de Basura (Pequeñas)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>T-Shirt Bag Lg.</t>
+          <t>Togo T-Shirt Bag Lg.</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Bolsa tipo camiseta grande</t>
+          <t>Bolsa tipo Camiseta para Llevar G</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>T-Shirt Bag Med</t>
+          <t>Togo T-Shirt Bag Med</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Bolsa tipo camiseta mediana</t>
+          <t>Bolsa tipo Camiseta para Llevar M</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>T-Shirt Bag Sm</t>
+          <t>Togo T-Shirt Bag Sm</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Bolsa tipo camiseta pequeña</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Cake Pan w/Lid</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Molde para pastel con tapa</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Cake Pan rounds</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Moldes redondos para pastel</t>
+          <t>Bolsa tipo Camiseta para Llevar P</t>
         </is>
       </c>
     </row>
@@ -2944,300 +2323,300 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>l1: English</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>l2: Español</t>
+          <t>es</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>@category: Frozen &amp; Refrigerated</t>
+          <t>FROZEN.REF</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>@category: Frozen &amp; Refrigerated</t>
+          <t>FROZEN.REF</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Biscuits 1/24 cs.</t>
+          <t>Cake Bundt</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Biscuits 1/24 caja</t>
+          <t>Pastel Bundt</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cake Bundt</t>
+          <t>Cake Chocolate</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pastel bundt</t>
+          <t>Pastel de Chocolate</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cake Chocolate</t>
+          <t>Cake Italian Lemon</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Pastel de chocolate</t>
+          <t>Pastel de Limón Italiano</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Cake Italian Lemon Crème</t>
+          <t>Cake Strawberry</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pastel italiano de limón crème</t>
+          <t>Pastel de Fresa</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cake Strawberry</t>
+          <t>Cannoli Cream w/choc</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Pastel de fresa</t>
+          <t>Crema de Cannoli con Chocolate</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cannoli Cream w/choc</t>
+          <t>Cannoli Shell Lg</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Crema de cannoli con chocolate</t>
+          <t>Concha de Cannoli Grande</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cannoli Shell Lg</t>
+          <t>Cannoli Shell Lg (choc)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Concha de cannoli grande</t>
+          <t>Concha de Cannoli Grande (Choc)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cannoli Shell Lg (choc)</t>
+          <t>Cannoli Shell Sm</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Concha de cannoli grande (chocolate)</t>
+          <t>Concha de Cannoli Pequeña</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Cannoli Shell Sm</t>
+          <t>Cannoli Shell Sm (choc)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Concha de cannoli pequeña</t>
+          <t>Concha de Cannoli Pequeña (Choc)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cannoli Shell Sm (choc)</t>
+          <t>Cheesecake NY</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Concha de cannoli pequeña (chocolate)</t>
+          <t>Pastel de Queso estilo NY</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cheesecake NY</t>
+          <t>Cheesecake Oreo</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cheesecake estilo Nueva York</t>
+          <t>Pastel de Queso Oreo</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cheesecake Oreo</t>
+          <t>Cheesecake Turtle</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cheesecake de Oreo</t>
+          <t>Pastel de Queso Tortuga</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cheesecake Turtle</t>
+          <t>French Fries Crinkle Cut</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cheesecake Turtle</t>
+          <t>Papas Fritas Onduladas</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>French Fries 3/8th" Straight</t>
+          <t>French Fries Homestyle</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Papas fritas rectas de 3/8"</t>
+          <t>Papas Fritas Estilo Casero</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>French Fries Crinkle Cut</t>
+          <t>French Fries Shoestring</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Papas fritas corte ondulado</t>
+          <t>Papas Fritas Finas</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>French Fries Homestyle</t>
+          <t>Hashbrown 2/10lb.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Papas fritas estilo casero</t>
+          <t>Papas Ralladas (Hashbrown) 2/10lb.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>French Fries Shoestring</t>
+          <t>Pasta Tortellini</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Papas fritas tipo shoestring</t>
+          <t>Pasta Tortellini</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Hashbrown 2/10lb.</t>
+          <t>Pizza Crust Cauliflower</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Hashbrown 2/10 lb.</t>
+          <t>Masa de Pizza de Coliflor</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Pasta Tortellini</t>
+          <t>Tater Tots</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Pasta tortellini</t>
+          <t>Croquetas de Papa (Tater Tots)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Pizza Crust Cauliflower</t>
+          <t>Tiramisu (ea.)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Base de pizza de coliflor</t>
+          <t>Tiramisú (c/u)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Tater Tots</t>
+          <t>French Fries 3/8th" Straight</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Tater tots</t>
+          <t>Papas Fritas Rectas 3/8"</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Tiramisu (ea.)</t>
+          <t>Biscuits 1/24 cs.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tiramisú (unidad)</t>
+          <t>Panecillos 1/24 caja</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Tortillas Chips uncooked</t>
+          <t> </t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Totopos sin cocinar</t>
+          <t> </t>
         </is>
       </c>
     </row>
@@ -3252,726 +2631,606 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B60"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>l1: English</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>l2: Español</t>
+          <t>es</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>@category: Dry Grocery</t>
+          <t>GROCERY DRY</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>@category: Dry Grocery</t>
+          <t>GROCERY DRY</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Banana Peppers sliced 1gal.</t>
+          <t>Baguettes</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Chiles banana rebanados 1 gal.</t>
+          <t>Baguettes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Barbecue Sauce 1 gal.</t>
+          <t>Basalmic Glaze</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Salsa barbecue 1 gal.</t>
+          <t>Glaseado Balsámico</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Basalmic Glaze</t>
+          <t>Bread Crumbs Panko 25lb.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Glaseado balsámico</t>
+          <t>Pan Rallado Panko 25lb.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Black Olives Sliced #10 can/cs.</t>
+          <t>Bread Sliced Sandwich</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Aceitunas negras rebanadas lata #10/caja</t>
+          <t>Pan de Molde en Rebanadas</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bread Baguettes</t>
+          <t>Buns Hamburger</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Baguettes</t>
+          <t>Pan para Hamburguesas</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bread Brioche Buns</t>
+          <t>Buns Hot Dog</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Pan brioche para hamburguesa</t>
+          <t>Pan para Hot Dogs</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Bread Crumbs Panko 25lb.</t>
+          <t>Croutons 4/2.5lbs.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pan molido panko 25 lb.</t>
+          <t>Crutones 4/2.5lbs.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Bread Hawaiian</t>
+          <t>Dressing Caesar 1 gal</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pan hawaiano</t>
+          <t>Aderezo César 1 galón</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bread Sliced Sandwich</t>
+          <t>Dressing Italian 1 gal.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Pan de sándwich rebanado</t>
+          <t>Aderezo Italiano 1 galón</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Brown Sugar 1lb.</t>
+          <t>Dressing Mix Italian packet</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Azúcar morena 1 lb.</t>
+          <t>Mezcla de Aderezo Italiano en paquete</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Buns Hamburger</t>
+          <t>Dressing Mix Ranch packet</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Pan para hamburguesa</t>
+          <t>Mezcla de Aderezo Ranchero en paquete</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Buns Hot Dog</t>
+          <t>Dressing Vinagrette 1 gal.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pan para hot dog</t>
+          <t>Vinagreta 1 galón</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Chocolate for Cannoli #10 can</t>
+          <t>Flour High Gluten All Trump 25lb.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Chocolate para cannoli lata #10</t>
+          <t>Harina de Alto Gluten All Trump 25lb.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Cole Slaw Dressing 1gal.</t>
+          <t>Flour High Gluten All Trump 50lb.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Aderezo para cole slaw 1 gal.</t>
+          <t>Harina de Alto Gluten All Trump 50lb.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Cole Slaw mix bag</t>
+          <t>Tortillas Flour 10"</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bolsa de mezcla para cole slaw</t>
+          <t>Tortillas de Harina 10"</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Croutons 4/2.5lbs.</t>
+          <t>Fry Oil</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Crutones 4/2.5 lb.</t>
+          <t>Aceite para Freír</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Dressing Caesar 1 gal</t>
+          <t>Garlic Minced in water</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Aderezo César 1 gal.</t>
+          <t>Ajo Picado en agua</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dressing Italian 1 gal.</t>
+          <t>Garlic Powder 5lb.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Aderezo italiano 1 gal.</t>
+          <t>Ajo en Polvo 5lb.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Dressing Mix Italian packet</t>
+          <t>Hot Sauce Red Hot 1 gal.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Mezcla para aderezo italiano, sobre</t>
+          <t>Salsa Picante Red Hot 1 galón</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Dressing Mix Ranch cs.</t>
+          <t>Jalapeno Sliced #10</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Mezcla para aderezo ranch (caja)</t>
+          <t>Jalapeño en Rodajas lata #10</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Dressing Mix Ranch packet</t>
+          <t>Mayonnaise 4/1 gal.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mezcla para aderezo ranch, sobre</t>
+          <t>Mayonesa 4/1 galón</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Dressing Vinagrette 1 gal.</t>
+          <t xml:space="preserve">Olive Ripe Sliced #10 </t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Vinagreta 1 gal.</t>
+          <t xml:space="preserve">Aceitunas Maduras en Rodajas lata #10 </t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Everything Bagel</t>
+          <t>Onion minced dried</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Bagel everything</t>
+          <t>Cebolla Picada Seca</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Flour High Gluten All Trump 25lb.</t>
+          <t>Onion Powder</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Harina alta en gluten All Trump 25 lb.</t>
+          <t>Cebolla en Polvo</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Flour High Gluten All Trump 50lb.</t>
+          <t>Pan Spray cs</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Harina alta en gluten All Trump 50 lb.</t>
+          <t>Aerosol para Sartén caja</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Fry Oil</t>
+          <t>Parmesan Packets</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Aceite para freír</t>
+          <t>Paquetes de Queso Parmesano</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Garlic Minced in water</t>
+          <t>Parsley minced dried</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Ajo picado en agua</t>
+          <t>Perejil Picado Seco</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Garlic Powder 5lb.</t>
+          <t>Pasta Fettucine 10"</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ajo en polvo 5 lb.</t>
+          <t>Pasta Fettuccine 10"</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Hot Sauce Red Hot 1 gal.</t>
+          <t>Pasta Lasagna 10"</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Salsa picante Red Hot 1 gal.</t>
+          <t>Pasta Lasaña 10"</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Jalapeno Sliced #10</t>
+          <t>Pasta Penne Rigate</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Jalapeño rebanado #10</t>
+          <t>Pasta Penne Rigate</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Mayonnaise 4/1 gal.</t>
+          <t>Pasta Rotini Tri Color</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Mayonesa 4/1 gal.</t>
+          <t>Pasta Rotini Tricolor</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Olive Ripe Sliced #10</t>
+          <t>Pasta Spaghetti 10"</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Aceituna madura rebanada #10</t>
+          <t>Pasta Espagueti 10"</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Onion minced dried</t>
+          <t>Pepperoncini Whole 1 gal.</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cebolla seca picada</t>
+          <t>Pepperoncini Entero 1 galón</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Onion Powder</t>
+          <t>Pineapple tidbits #10</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Cebolla en polvo</t>
+          <t>Trozos de Piña lata #10</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Oreos pkg.</t>
+          <t>Ranch Dressing mix cs.</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Galletas Oreo, paquete</t>
+          <t>Mezcla para Aderezo Ranchero caja</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Packets Parmesan</t>
+          <t>Red Pepper Packets</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Sobres de parmesano</t>
+          <t>Paquetes de Chile Rojo</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Packets Red Pepper cs.</t>
+          <t>Salsa Fire Roasted #10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Sobres de chile rojo (caja)</t>
+          <t>Salsa Asada al Fuego lata #10</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Pan Spray cs</t>
+          <t>Salt 50lb.</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Spray para sartén (caja)</t>
+          <t>Sal 50lb.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Parsley minced dried</t>
+          <t>Sugar 50lb.</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Perejil seco picado</t>
+          <t>Azúcar 50lb.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Pasta Fettucine 10"</t>
+          <t>Tomato Paste cs.</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Pasta fettuccine 10"</t>
+          <t>Pasta de Tomate caja</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Pasta Lasagna 10"</t>
+          <t>Tomato Sauce cs.</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Pasta para lasaña 10"</t>
+          <t>Salsa de Tomate caja</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Pasta Penne Rigate</t>
+          <t>Vinegar Red 1 gal</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Pasta penne rigate</t>
+          <t>Vinagre Tinto 1 galón</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Pasta Rotini Tri Color</t>
+          <t>Vinegar White 1 gal</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Pasta rotini tricolor</t>
+          <t>Vinagre Blanco 1 galón</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Pasta Spaghetti 10"</t>
+          <t xml:space="preserve">Yeast </t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Pasta espagueti 10"</t>
+          <t>Levadura</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Pepperoncini Whole 1 gal.</t>
+          <t>Chocolate for Cannoli #10 can</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Pepperoncini entero 1 gal.</t>
+          <t>Chocolate para Cannoli lata #10</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Pineapple tidbits #10</t>
+          <t>Texas Toast</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Piña en trozos #10</t>
+          <t>Tostada Texana</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Plain Bagel</t>
+          <t>Everything Bagel</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Bagel natural</t>
+          <t>Bagel Todo (Everything)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Salsa Fire Roasted #10</t>
+          <t>Plain Bagel</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Salsa fire roasted #10</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Salt 50lb.</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Sal 50 lb.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Sugar 50lb.</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Azúcar 50 lb.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Sugar Powdered bag</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Azúcar glass, bolsa</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Texas Toast</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Texas toast</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Tomato Paste cs.</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Pasta de tomate (caja)</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Tomato Sauce cs.</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Salsa de tomate (caja)</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Tortillas Flour 10"</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Tortillas de harina 10"</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Vinegar Red 1 gal</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Vinagre rojo 1 gal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Vinegar White 1 gal</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Vinagre blanco 1 gal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Yeast</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Levadura</t>
+          <t>Bagel Sencillo</t>
         </is>
       </c>
     </row>
@@ -3992,240 +3251,240 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>l1: English</t>
+          <t>en</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>l2: Español</t>
+          <t>es</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>@category: Meats</t>
+          <t>MEATS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>@category: Carnes</t>
+          <t>Carnes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bacon Bits (case)</t>
+          <t>Bacon Sliced 1cs</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tocino en trocitos (caja)</t>
+          <t>Tocino en Rebanadas 1 caja</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bacon Sliced 1cs</t>
+          <t>Canadian Bacon</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tocino rebanado 1 caja</t>
+          <t>Tocino Canadiense</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Brisket (each)</t>
+          <t>Ground Beef 73/27 lbs</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Brisket (unidad)</t>
+          <t>Carne Molida 73/27 lbs</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Canadian Bacon (case)</t>
+          <t>Ground Beef 80/20 lbs</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tocino canadiense (caja)</t>
+          <t>Carne Molida 80/20 lbs</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Catfish/Swai cs.</t>
+          <t>Ground Beef 90/10 lbs</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bagre/Swai (caja)</t>
+          <t>Carne Molida 90/10 lbs</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Chicken Breast (case)</t>
+          <t>Italian Sausage Rope</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Pechuga de pollo (caja)</t>
+          <t>Salchicha Italiana en Cuerda</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Chicken Wings (case)</t>
+          <t>Pepperoni</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alitas de pollo (caja)</t>
+          <t>Pepperoni</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ground Beef 73/27 lbs</t>
+          <t>Philly Meat</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Carne molida 73/27 lb.</t>
+          <t>Carne para Philly</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ground Beef 80/20 lbs</t>
+          <t>Chicken Breast</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Carne molida 80/20 lb.</t>
+          <t>Pechuga de Pollo</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Ground Beef 90/10 lbs</t>
+          <t>Chicken Wings</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Carne molida 90/10 lb.</t>
+          <t>Alitas de Pollo</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Hot Dogs (each)</t>
+          <t xml:space="preserve">Bacon Bits </t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hot dogs (unidad)</t>
+          <t xml:space="preserve">Trozos de Tocino </t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Hot Links (each)</t>
+          <t>Shrimp 21-25 raw peeled 5/2lb.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Salchichas hot links (unidad)</t>
+          <t>Camarones 21-25 crudos y pelados 5/2lb.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Italian Sausage Rope (case)</t>
+          <t>Brisket</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Salchicha italiana en tira (caja)</t>
+          <t>Pecho de Res (Brisket)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Pepperoni (case)</t>
+          <t>Pork Butt</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Pepperoni (caja)</t>
+          <t>Paleta de Cerdo</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Philly Meat (case)</t>
+          <t>Polish Sausage</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Carne tipo Philly (caja)</t>
+          <t>Salchicha Polaca</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Polish Sausage (each)</t>
+          <t>Hot Links</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Salchicha polaca (unidad)</t>
+          <t>Salchichas Picantes</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Pork Butt (each)</t>
+          <t>Hot Dogs</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Pork butt (unidad)</t>
+          <t>Hot Dogs</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Shrimp 21-25 raw peeled 5/2lb. (case)</t>
+          <t>Catfish/Swai cs.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Camarón 21-25 crudo pelado 5/2 lb. (caja)</t>
+          <t>Bagre/Swai caja</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "docs: update master inventory format guide and master sheet"
</commit_message>
<xml_diff>
--- a/item master/Master.xlsx
+++ b/item master/Master.xlsx
@@ -7,19 +7,18 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="BEV-ALC" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="BEV-BIB" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="BEV-RTD" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="CLEANING" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="DAIRY" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="DISPOSABLES" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="FROZEN.REF" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="GROCERY DRY" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MEATS" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="PRODUCE" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="PREPARED" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="SMALLWARES" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="BAKERY" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Alcohol (🍺)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fountain BIB (🧃)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Beverages (🥤)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cleaning (🧹)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Dairy (🧀)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Disposables (🥡)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Frozen &amp; Refrigerated (❄️)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Dry Grocery (🌾)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Meats (🥩)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Produce (🥦)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Prepared (🍲)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Smallwares (🍴)" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,114 +424,450 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>l1: English</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>l2: Español</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BEV-ALC</t>
+          <t>@category: Alcohol</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BEV-ALC</t>
+          <t>@category: Alcohol</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Stella Artois 6pk</t>
+          <t>Blue Moon 6pk.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Stella Artois 6pk</t>
+          <t>Blue Moon 6 paquetes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Yuengling Flight 6pk</t>
+          <t>Bud Light 6pk</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yuengling Flight 6pk</t>
+          <t>Bud Light 6 paquetes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Bud Light 6pk</t>
+          <t>Budweiser 6pk.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bud Light 6pk</t>
+          <t>Budweiser 6 paquetes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Modelo Negra 6pk</t>
+          <t>Coors Light 6pk.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Modelo Negra 6pk</t>
+          <t>Coors Light 6 paquetes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>F5 IPA 6pk</t>
+          <t>Corona 6pk</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>F5 IPA 6pk</t>
+          <t>Corona 6 paquetes</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Corona 6pk</t>
+          <t>Fat Tire Ale 6pk.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Corona 6pk</t>
+          <t>Fat Tire Ale 6 paquetes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Heineken 6pk.</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Heineken 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Heineken Zero 6pk.</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Heineken Zero 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>IPA DNR 6pk.</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>IPA DNR 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>IPA F5 6pk</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>IPA F5 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>IPA Native Amber</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>IPA Native Amber</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Michelob Ultra 6pk.</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Michelob Ultra 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Michelob Ultra Zero 6pk.</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Michelob Ultra Zero 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Miller Lite 6pk.</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Miller Lite 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Modelo 6pk.</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Modelo 6pk.</t>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Modelo 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Modelo Negra 6pk</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Modelo Negra 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Peroni 6pk.</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Peroni 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Sam Adams Lager</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Sam Adams Lager</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Shiner Bock 6pk.</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Shiner Bock 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Shock Top 6pk.</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Shock Top 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Stella Artois 6pk</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Stella Artois 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Truly Cherry</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Truly cereza</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Truly Strawberry Lime</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Truly fresa-limón</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>XX Chelada 6pk.</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>XX Chelada 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>XX Lager 6pk.</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>XX Lager 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>XX Lager Dark 6pk.</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>XX Lager Dark 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Yuengling Flight 6pk</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Yuengling Flight 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Yuengling Lager 6pk</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Yuengling Lager 6 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Apothic Red</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Apothic Red</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Bread &amp; Butter Pinot Noir</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Bread &amp; Butter Pinot Noir</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Gabbiano Chianti</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Gabbiano Chianti</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Gallo .187 Cabernet Sauvignon 4pk.</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Gallo .187 Cabernet Sauvignon 4 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Josh Cabernet Sauvignon</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Josh Cabernet Sauvignon</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Sutter Home .187 Sauvignon Blanc 4pk.</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Sutter Home .187 Sauvignon Blanc 4 paquetes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Yellowtail Pinot Noir</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Yellowtail Pinot Noir</t>
         </is>
       </c>
     </row>
@@ -547,90 +882,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>l1: English</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>l2: Español</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PRODUCE</t>
+          <t>@category: Produce</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Productos Frescos</t>
+          <t>@category: Productos Frescos</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Basil Fresh</t>
+          <t>Basil Fresh (each)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Albahaca Fresca</t>
+          <t>Albahaca fresca (unidad)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bell Peppers (Yellow, Red,Orange) 6 pk</t>
+          <t>Bell Peppers (Yellow, Red,Orange) 6 pk (each)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pimientos (Amarillo, Rojo, Naranja) 6 paq.</t>
+          <t>Pimientos morrones (amarillo, rojo, naranja) paquete de 6 (unidad)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Bell Peppers Choppers</t>
+          <t>Bell Peppers Choppers (case)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Pimientos para Picar</t>
+          <t>Pimientos morrones picados (caja)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Broccoli Florets (fresh)</t>
+          <t>Broccoli Florets (fresh) (case)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Flores de Brócoli (frescas)</t>
+          <t>Floretes de brócoli (fresco) (caja)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Broccoli Florets (frozen)</t>
+          <t>Broccoli Florets (frozen) (case)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Flores de Brócoli (congeladas)</t>
+          <t>Floretes de brócoli (congelado) (caja)</t>
         </is>
       </c>
     </row>
@@ -649,120 +984,132 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Constellation Cherry Tomatoes</t>
+          <t>Cucumber English 2 pk (each)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tomates Cherry Constellation</t>
+          <t>Pepino inglés paquete de 2 (unidad)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cucumber English 2 pk</t>
+          <t>Lettuce Romaine (case)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pepino Inglés 2 paq.</t>
+          <t>Lechuga romana (caja)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Lettuce Romaine</t>
+          <t>Mushroom Medium (case)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lechuga Romana</t>
+          <t>Champiñón mediano (caja)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mushroom Medium</t>
+          <t>Onion Red (case)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Champiñones Medianos</t>
+          <t>Cebolla roja (caja)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Onion Red</t>
+          <t>Onion Yellow (case)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cebolla Roja</t>
+          <t>Cebolla amarilla (caja)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Onion Yellow</t>
+          <t>Potato Idaho 70 ct./50 lb. (case)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cebolla Amarilla</t>
+          <t>Papa Idaho 70 ct./50 lb. (caja)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Potato Idaho 70 ct./50 lb.</t>
+          <t>Spinach Fresh (each)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Papas Idaho 70 ct./50 lb.</t>
+          <t>Espinaca fresca (unidad)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Spinach Fresh</t>
+          <t>Tomato Cherry (case)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Espinaca Fresca</t>
+          <t>Tomate cherry (caja)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Tomato Cherry</t>
+          <t>Tomato Cherry Constellation (each)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tomates Cherry</t>
+          <t>Tomate cherry Constellation (unidad)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Tomato Roma</t>
+          <t>Tomato Roma (each)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tomates Roma</t>
+          <t>Tomate Roma (unidad)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Tomato Slicer (case)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Tomate para rebanar (caja)</t>
         </is>
       </c>
     </row>
@@ -783,252 +1130,252 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>l1: English</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>l2: Español</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PREPARED</t>
+          <t>@category: Prepared</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PREPARED</t>
+          <t>@category: Prepared</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Chicken Breast Cooked (4 oz.)</t>
+          <t>Bacon Bits (qt) (each)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Pechuga de Pollo Cocida (4 oz.)</t>
+          <t>Trocitos de tocino (cuarto) (unidad)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Boneless Bites (prepared 8 ea.)</t>
+          <t>Bell Pepper Chopped (qt.) (each)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Trozos sin Hueso (preparados 8 c/u)</t>
+          <t>Pimiento morrón picado (cuarto) (unidad)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Chicken Tenders (prepared 3 ea.)</t>
+          <t>Boneless Bites (prepared 8 ea.)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tiras de Pollo (preparadas 3 c/u)</t>
+          <t>Boneless preparados (8 pzas.)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dough Par Bake 18"</t>
+          <t>Chicken Breast Cooked (4 oz.) (each)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Masa Pre-cocida 18"</t>
+          <t>Pechuga de pollo cocida (4 oz.) (unidad)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Marinara (gal.)</t>
+          <t>Chicken Parmesan (prepared) ea.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Salsa Marinara (gal.)</t>
+          <t>Pollo parmesano (preparado) unidad</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pizza Sauce (gal.)</t>
+          <t>Chicken Tenders (prepared 3 ea.)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Salsa de Pizza (gal.)</t>
+          <t>Tiras de pollo (preparadas, 3 pzas.)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Italian Sausage Cooked (lb.)</t>
+          <t>Dough Par Bake 18" (each)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Salchicha Italiana Cocida (lb.)</t>
+          <t>Masa prehorneada 18" (unidad)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Onion Diced (qt.)</t>
+          <t>Fettucine Alfredo (prepared) ea.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cebolla Cortada en Cubitos (cto.)</t>
+          <t>Fettuccine Alfredo (preparado) unidad</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Onion Sliced (qt.)</t>
+          <t>Italian Sausage Cooked (lb.) (each)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cebolla en Rodajas (cto.)</t>
+          <t>Salchicha italiana cocida (lb.) (unidad)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bell Pepper Chopped (qt.)</t>
+          <t>Marinara (gal.) (each)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pimiento Picado (cto.)</t>
+          <t>Marinara (galón) (unidad)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mushroom Sliced (qt)</t>
+          <t>Meatballs (ea)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Champiñones en Rodajas (cto.)</t>
+          <t>Albóndigas (unidad)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Tomatos Sliced (qt.)</t>
+          <t>Mushroom Sliced (qt) (each)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Tomates en Rodajas (cto.)</t>
+          <t>Champiñón rebanado (cuarto) (unidad)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Tomatos Diced (qt.)</t>
+          <t>Onion Diced (qt.) (each)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tomates Cortados en Cubitos (cto.)</t>
+          <t>Cebolla en cubos (cuarto) (unidad)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Bacon Bits (qt)</t>
+          <t>Onion Sliced (qt.) (each)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Trozos de Tocino (cto.)</t>
+          <t>Cebolla rebanada (cuarto) (unidad)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Stromboli (prepared) ea.</t>
+          <t>Pizza Sauce (gal.) (each)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Stromboli (preparado) c/u</t>
+          <t>Salsa para pizza (galón) (unidad)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Meatballs (ea)</t>
+          <t>Spaghetti w/meatballs (prepared) ea.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Albóndigas (c/u)</t>
+          <t>Espagueti con albóndigas (preparado) unidad</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Fettucine Alfredo (prepared) ea.</t>
+          <t>Stromboli (prepared) ea.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Fettuccine Alfredo (preparado) c/u</t>
+          <t>Stromboli (preparado) unidad</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Spaghetti w/meatballs (prepared) ea.</t>
+          <t>Tomatos Diced (qt.) (each)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Espaguetis con Albóndigas (preparado) c/u</t>
+          <t>Tomates en cubos (cuarto) (unidad)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Chicken Parmesan (prepared) ea.</t>
+          <t>Tomatos Sliced (qt.) (each)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Pollo a la Parmesana (preparado) c/u</t>
+          <t>Tomates rebanados (cuarto) (unidad)</t>
         </is>
       </c>
     </row>
@@ -1049,24 +1396,24 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>l1: English</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>l2: Español</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SMALLWARES</t>
+          <t>@category: Smallwares</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SMALLWARES</t>
+          <t>@category: Smallwares</t>
         </is>
       </c>
     </row>
@@ -1078,57 +1425,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Queseros</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>es</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>BAKERY</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>BAKERY</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Film Poly 24" Wrap</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Envoltura de Película Plástica 24"</t>
+          <t>Agitadores para queso</t>
         </is>
       </c>
     </row>
@@ -1149,24 +1446,24 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>l1: English</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>l2: Español</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BEV-BIB</t>
+          <t>@category: Fountain BIB</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BEV-BIB</t>
+          <t>@category: Fountain BIB</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1475,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Caja de Jarabe Coca-Cola</t>
+          <t>BIB Coca-Cola</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1487,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Caja de Jarabe Coke Zero</t>
+          <t>BIB Coke Zero</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1499,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Caja de Jarabe Diet Coke</t>
+          <t>BIB Diet Coke</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1511,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Caja de Jarabe Diet Dr. Pepper</t>
+          <t>BIB Diet Dr. Pepper</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1523,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Caja de Jarabe Dr. Pepper</t>
+          <t>BIB Dr Pepper</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1535,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Caja de Jarabe Limonada</t>
+          <t>BIB limonada</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1547,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Caja de Jarabe Cerveza de Raíz</t>
+          <t>BIB root beer</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1559,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Caja de Jarabe Sprite</t>
+          <t>BIB Sprite</t>
         </is>
       </c>
     </row>
@@ -1277,78 +1574,330 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>l1: English</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>l2: Español</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BEV-RTD</t>
+          <t>@category: Beverages</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BEV-RTD</t>
+          <t>@category: Beverages</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tea automatic brew 32/3.5oz.</t>
+          <t>Btl Gold Peak Tea Unsweet</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Té preparado automático 32/3.5oz.</t>
+          <t>Botella de té Gold Peak sin azúcar</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jarritos Asst Flavors cs.</t>
+          <t>Btl Henry Winehard Root Beer</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Jarritos Sabores Surtidos caja</t>
+          <t>Botella Henry Winehard root beer</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Mexican Coca-Cola cs</t>
+          <t>Btl Henry Winehard Vanilla Cream</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Coca-Cola Mexicana caja</t>
+          <t>Botella Henry Winehard vanilla cream</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mexican Sprite cs</t>
+          <t>Btl Jarritos Asst Flavors cs.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sprite Mexicano caja</t>
+          <t>Botella Jarritos sabores surtidos (caja)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Btl Mexican Coca-Cola cs</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Botella Coca-Cola mexicana (caja)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Btl Mexican Sprite cs</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Botella Sprite mexicano (caja)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Btl Pellegrino Ciao Lime</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Botella Pellegrino Ciao lima</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Btl Pellegrino Ciao Orange</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Botella Pellegrino Ciao naranja</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Btl Pellegrino Mineral Water</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Botella de agua mineral Pellegrino</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Btl Topo-Chico Lime</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Botella Topo-Chico lima</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Btl Topo-Chico Original</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Botella Topo-Chico original</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Btl Water</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Botella de agua</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Can A&amp;W Root Beer</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Lata A&amp;W root beer</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Can Coca-Cola</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Lata de Coca-Cola</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Can Diet Coke</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Lata de Diet Coke</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Can Diet Dr Pepper</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Lata de Diet Dr Pepper</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Can Dr Pepper</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Lata de Dr Pepper</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Can Grape Crush</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Lata de Crush de uva</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Can Mountain Dew</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Lata de Mountain Dew</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Can Okolo-Homa Cream Soda</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Lata Okolo-Homa cream soda</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Can Okolo-Homa Root Beer</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Lata Okolo-Homa root beer</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Can Orange Fanta</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Lata de Fanta naranja</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Can Pepsi</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Lata de Pepsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Can Sprite</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Lata de Sprite</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Tea automatic brew 32/3.5oz.</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Té para preparación automática 32/3.5 oz.</t>
         </is>
       </c>
     </row>
@@ -1363,30 +1912,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>l1: English</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>l2: Español</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CLEANING</t>
+          <t>@category: Cleaning</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CLEANING</t>
+          <t>@category: Cleaning</t>
         </is>
       </c>
     </row>
@@ -1405,12 +1954,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dish Detergent (dawn) </t>
+          <t>Dish Detergent (dawn)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Detergente para Platos (Dawn)</t>
+          <t>Detergente para platos (Dawn)</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1971,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Limpiador de Pisos (Fabuloso morado)</t>
+          <t>Limpiador de pisos (Fabuloso morado)</t>
         </is>
       </c>
     </row>
@@ -1434,7 +1983,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Esponjas de Acero Inoxidable 12/1 ct.</t>
+          <t>Fibra de acero inoxidable 12/1 ct.</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1995,43 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Desinfectante para Comedor</t>
+          <t>Sanitizante para comedor</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Stainless Steel cleaner</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Limpiador para acero inoxidable</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Magic Eraser</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Borrador mágico</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Window cleaner</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Limpiavidrios</t>
         </is>
       </c>
     </row>
@@ -1461,234 +2046,246 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>l1: English</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>l2: Español</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DAIRY</t>
+          <t>@category: Dairy</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Lácteos</t>
+          <t>@category: Lácteos</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Butter European 36/1lb.</t>
+          <t>American Cheese Sliced White pkg.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Mantequilla Europea 36/1lb.</t>
+          <t>Queso americano blanco en rebanadas, paquete</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Butter Unsalted 36/1lb.</t>
+          <t>American Cheese Sliced Yellow pkg.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mantequilla sin Sal 36/1lb.</t>
+          <t>Queso americano amarillo en rebanadas, paquete</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Buttermilk 1cs.</t>
+          <t>Butter European 36/1lb.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Suero de Mantequilla 1 caja</t>
+          <t>Mantequilla europea 36/1 lb.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Cream Cheese 10/3lb.</t>
+          <t>Butter Unsalted 36/1lb.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Queso Crema 10/3lb.</t>
+          <t>Mantequilla sin sal 36/1 lb.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Eggs 15 doz.</t>
+          <t>Buttermilk 1cs.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Huevos 15 docenas</t>
+          <t>Suero de leche 1 caja</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Heavy Cream cs.</t>
+          <t>Cream Cheese 10/3lb.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Crema Espesa caja</t>
+          <t>Queso crema 10/3 lb.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mozzarella BelGioioso Fresh 2/1lb.</t>
+          <t>Eggs 15 doz.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mozzarella Fresca BelGioioso 2/1lb.</t>
+          <t>Huevos 15 docenas</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mozzarella Loaf 8/6lb.</t>
+          <t>Heavy Cream cs.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Barra de Mozzarella 8/6lb.</t>
+          <t>Crema espesa (caja)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mozzarella Shredded 5lb.</t>
+          <t>Mozzarella BelGioioso Fresh 2/1lb.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mozzarella Rallada 5lb.</t>
+          <t>Mozzarella fresca BelGioioso 2/1 lb.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Parmesan Grated 5lb.</t>
+          <t>Mozzarella Loaf 8/6lb.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Parmesano Rallado 5lb.</t>
+          <t>Mozzarella tipo loaf 8/6 lb.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Parmesan Shredded 5lb.</t>
+          <t>Mozzarella Shredded 5lb.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Parmesano en Hebras 5lb.</t>
+          <t>Mozzarella rallada 5 lb.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ricotta Cheese 6/3lb.</t>
+          <t>Parmesan Grated 5lb.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Queso Ricotta 6/3lb.</t>
+          <t>Parmesano rallado 5 lb.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sour Cream 4/5lb.</t>
+          <t>Parmesan Shredded 5lb.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Crema Agria 4/5lb.</t>
+          <t>Parmesano deshebrado 5 lb.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sour Cream packets</t>
+          <t>Provolone sliced pkg.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Paquetes de Crema Agria</t>
+          <t>Provolone en rebanadas, paquete</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Provolone sliced pkg.</t>
+          <t>Ricotta Cheese 6/3lb.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Provolone en Rebanadas paq.</t>
+          <t>Queso ricotta 6/3 lb.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>American Cheese Sliced Yellow pkg.</t>
+          <t>Sour Cream 4/5lb.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Queso Americano Amarillo Rebanado paq.</t>
+          <t>Crema agria 4/5 lb.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>American Cheese Sliced White pkg.</t>
+          <t>Sour Cream packets</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Queso Americano Blanco Rebanado paq.</t>
+          <t>Sobres de crema agria</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Cheddar Cheese Shredded 5lb.</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Queso cheddar rallado 5 lb.</t>
         </is>
       </c>
     </row>
@@ -1703,30 +2300,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>l1: English</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>l2: Español</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DISPOSABLES</t>
+          <t>@category: Disposables</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DISPOSABLES</t>
+          <t>@category: Disposables</t>
         </is>
       </c>
     </row>
@@ -1738,7 +2335,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Plato de Papel Ultra 08"</t>
+          <t>Plato de papel Ultra Lunch de 8"</t>
         </is>
       </c>
     </row>
@@ -1750,7 +2347,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Plato de Papel Ultra 10"</t>
+          <t>Plato de papel Ultra Lunch de 10"</t>
         </is>
       </c>
     </row>
@@ -1762,7 +2359,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Vaso de Espuma 16 oz.</t>
+          <t>Vaso de espuma de 16 oz.</t>
         </is>
       </c>
     </row>
@@ -1774,7 +2371,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tapa para Vaso de Espuma 16 oz.</t>
+          <t>Tapa de espuma de 16 oz.</t>
         </is>
       </c>
     </row>
@@ -1786,7 +2383,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Vasito Transparente para Porción 2 oz.</t>
+          <t>Vaso transparente para porción de 2 oz.</t>
         </is>
       </c>
     </row>
@@ -1798,7 +2395,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tapa Transparente para Porción 2 oz.</t>
+          <t>Tapa transparente para porción de 2 oz.</t>
         </is>
       </c>
     </row>
@@ -1810,7 +2407,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Vasito de Espuma para Porción 4 oz.</t>
+          <t>Vaso de espuma para porción de 4 oz.</t>
         </is>
       </c>
     </row>
@@ -1822,7 +2419,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tapa de Espuma para Porción 4 oz.</t>
+          <t>Tapa de espuma para porción de 4 oz.</t>
         </is>
       </c>
     </row>
@@ -1834,31 +2431,31 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Envase de Plástico Transparente para Llevar 6x6</t>
+          <t>Contenedor plástico transparente 6x6 para llevar</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>8x8 Clear togo boxes cs</t>
+          <t>6x6 White Foam togo</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cajas Transparentes para Llevar 8x8 caja</t>
+          <t>Contenedor blanco de espuma 6x6 para llevar</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>6x6 White Foam togo</t>
+          <t>8x8 Clear togo boxes cs</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Envase de Espuma Blanca para Llevar 6x6</t>
+          <t>Cajas transparentes 8x8 para llevar (caja)</t>
         </is>
       </c>
     </row>
@@ -1870,7 +2467,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Envase de Espuma Blanca para Llevar 8x8</t>
+          <t>Contenedor blanco de espuma 8x8 para llevar</t>
         </is>
       </c>
     </row>
@@ -1882,7 +2479,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Envase de Espuma Blanca para Llevar 9x9</t>
+          <t>Contenedor blanco de espuma 9x9 para llevar</t>
         </is>
       </c>
     </row>
@@ -1894,7 +2491,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Rollo de Papel Aluminio</t>
+          <t>Rollo de papel aluminio</t>
         </is>
       </c>
     </row>
@@ -1906,19 +2503,19 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Hojas de Papel Aluminio 10.75" 1/200 ct.</t>
+          <t>Hojas de aluminio 10.75" 1/200 ct.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aluminum Lid (full Pan)</t>
+          <t>Aluminum Lid (FULL Pan)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tapa de Aluminio (Bandeja Completa)</t>
+          <t>Tapa de aluminio (charola completa)</t>
         </is>
       </c>
     </row>
@@ -1930,19 +2527,19 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Tapa de Aluminio (Media Bandeja)</t>
+          <t>Tapa de aluminio (media charola)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aluminum Pan (full pan)</t>
+          <t>Aluminum Pan (FULL pan)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bandeja de Aluminio (Completa)</t>
+          <t>Charola de aluminio (charola completa)</t>
         </is>
       </c>
     </row>
@@ -1954,271 +2551,271 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Bandeja de Aluminio (Media)</t>
+          <t>Charola de aluminio (media charola)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Cutlery Meal Kit</t>
+          <t>Cutlery Fork White Heavy Duty box</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Kit de Cubiertos para Comida</t>
+          <t>Caja de tenedores blancos resistentes</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Deli container togo 16oz.</t>
+          <t>Cutlery Knife White Heavy Duty box</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Envase Deli para Llevar 16 oz.</t>
+          <t>Caja de cuchillos blancos resistentes</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Deli container togo 8oz.</t>
+          <t>Cutlery Meal Kit</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Envase Deli para Llevar 8 oz.</t>
+          <t>Kit de cubiertos</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Deli container togo lids</t>
+          <t>Deli container togo 16oz.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Tapas para Envases Deli para Llevar</t>
+          <t>Contenedor deli para llevar de 16 oz.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Film Poly 12" Wrap</t>
+          <t>Deli container togo 8oz.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Envoltura de Película Plástica 12"</t>
+          <t>Contenedor deli para llevar de 8 oz.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Film Poly 18" Wrap</t>
+          <t>Deli container togo lids</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Envoltura de Película Plástica 18"</t>
+          <t>Tapas para contenedor deli para llevar</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Film Poly 24" Wrap</t>
+          <t>Dinner Knapkins</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Envoltura de Película Plástica 24"</t>
+          <t>Servilletas para comida</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Fork White Heavy Duty box</t>
+          <t>Film Poly 12" Wrap</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Tenedor Blanco de Alta Resistencia caja</t>
+          <t>Rollo de film plástico de 12"</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Gloves Lg</t>
+          <t>Film Poly 18" Wrap</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Guantes G</t>
+          <t>Rollo de film plástico de 18"</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Gloves Med</t>
+          <t>Film Poly 24" Wrap</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Guantes M</t>
+          <t>Rollo de film plástico de 24"</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Gloves Sm</t>
+          <t>Gloves Lg</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Guantes P</t>
+          <t>Guantes grandes</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Knife White Heavy Duty box</t>
+          <t>Gloves Med</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Cuchillo Blanco de Alta Resistencia caja</t>
+          <t>Guantes medianos</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Menu Tissue (sgl)</t>
+          <t>Gloves Sm</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Papel Seda para Menú (sgl)</t>
+          <t>Guantes pequeños</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Paper Towel (brown roll)</t>
+          <t>Menu Tissue (sgl)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Toalla de Papel (Rollo Marrón)</t>
+          <t>Papel para menú (individual)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Paper Towels (dispenser)</t>
+          <t>Paper Towel (brown roll)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Toallas de Papel (Dispensador)</t>
+          <t>Toalla de papel (rollo café)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Paper Towels (kitchen)</t>
+          <t>Paper Towels (dispenser)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Toallas de Papel (Cocina)</t>
+          <t>Toallas de papel (dispensador)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Pizza Boxes 10"</t>
+          <t>Paper Towels (kitchen)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Cajas de Pizza 10"</t>
+          <t>Toallas de papel (cocina)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Pizza Boxes 14"</t>
+          <t>Pizza Boxes 10"</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cajas de Pizza 14"</t>
+          <t>Cajas para pizza de 10"</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Pizza Boxes 18"</t>
+          <t>Pizza Boxes 14"</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Cajas de Pizza 18"</t>
+          <t>Cajas para pizza de 14"</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Portion Control Bag (sandwich size)</t>
+          <t>Pizza Boxes 18"</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Bolsa de Control de Porción (Tamaño Sándwich)</t>
+          <t>Cajas para pizza de 18"</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Register 3 1/8" Thermal Roll</t>
+          <t>Portion Control Bag (sandwich size)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Rollo Térmico para Registradora 3 1/8"</t>
+          <t>Bolsa de control de porción (tamaño sándwich)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Register paper 3 1/8" Thermal</t>
+          <t>Register 3 1/8" Thermal Roll</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Papel Térmico para Registradora 3 1/8"</t>
+          <t>Rollo térmico para caja 3 1/8"</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2827,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Papel Higiénico</t>
+          <t>Papel higiénico</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2839,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Bolsas de Basura (Tamaño Cocina)</t>
+          <t>Bolsas de basura (tamaño cocina)</t>
         </is>
       </c>
     </row>
@@ -2254,7 +2851,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Bolsas de Basura (Grandes 55-65 gal)</t>
+          <t>Bolsas de basura grandes (55-65 gal.)</t>
         </is>
       </c>
     </row>
@@ -2266,43 +2863,67 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Bolsas de Basura (Pequeñas)</t>
+          <t>Bolsas de basura pequeñas</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Togo T-Shirt Bag Lg.</t>
+          <t>T-Shirt Bag Lg.</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Bolsa tipo Camiseta para Llevar G</t>
+          <t>Bolsa tipo camiseta grande</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Togo T-Shirt Bag Med</t>
+          <t>T-Shirt Bag Med</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Bolsa tipo Camiseta para Llevar M</t>
+          <t>Bolsa tipo camiseta mediana</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Togo T-Shirt Bag Sm</t>
+          <t>T-Shirt Bag Sm</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Bolsa tipo Camiseta para Llevar P</t>
+          <t>Bolsa tipo camiseta pequeña</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Cake Pan w/Lid</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Molde para pastel con tapa</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Cake Pan rounds</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Moldes redondos para pastel</t>
         </is>
       </c>
     </row>
@@ -2323,300 +2944,300 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>l1: English</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>l2: Español</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FROZEN.REF</t>
+          <t>@category: Frozen &amp; Refrigerated</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FROZEN.REF</t>
+          <t>@category: Frozen &amp; Refrigerated</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cake Bundt</t>
+          <t>Biscuits 1/24 cs.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Pastel Bundt</t>
+          <t>Biscuits 1/24 caja</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cake Chocolate</t>
+          <t>Cake Bundt</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pastel de Chocolate</t>
+          <t>Pastel bundt</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cake Italian Lemon</t>
+          <t>Cake Chocolate</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Pastel de Limón Italiano</t>
+          <t>Pastel de chocolate</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Cake Strawberry</t>
+          <t>Cake Italian Lemon Crème</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pastel de Fresa</t>
+          <t>Pastel italiano de limón crème</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cannoli Cream w/choc</t>
+          <t>Cake Strawberry</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Crema de Cannoli con Chocolate</t>
+          <t>Pastel de fresa</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cannoli Shell Lg</t>
+          <t>Cannoli Cream w/choc</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Concha de Cannoli Grande</t>
+          <t>Crema de cannoli con chocolate</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cannoli Shell Lg (choc)</t>
+          <t>Cannoli Shell Lg</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Concha de Cannoli Grande (Choc)</t>
+          <t>Concha de cannoli grande</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cannoli Shell Sm</t>
+          <t>Cannoli Shell Lg (choc)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Concha de Cannoli Pequeña</t>
+          <t>Concha de cannoli grande (chocolate)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Cannoli Shell Sm (choc)</t>
+          <t>Cannoli Shell Sm</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Concha de Cannoli Pequeña (Choc)</t>
+          <t>Concha de cannoli pequeña</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cheesecake NY</t>
+          <t>Cannoli Shell Sm (choc)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pastel de Queso estilo NY</t>
+          <t>Concha de cannoli pequeña (chocolate)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cheesecake Oreo</t>
+          <t>Cheesecake NY</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Pastel de Queso Oreo</t>
+          <t>Cheesecake estilo Nueva York</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cheesecake Turtle</t>
+          <t>Cheesecake Oreo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pastel de Queso Tortuga</t>
+          <t>Cheesecake de Oreo</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>French Fries Crinkle Cut</t>
+          <t>Cheesecake Turtle</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Papas Fritas Onduladas</t>
+          <t>Cheesecake Turtle</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>French Fries Homestyle</t>
+          <t>French Fries 3/8th" Straight</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Papas Fritas Estilo Casero</t>
+          <t>Papas fritas rectas de 3/8"</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>French Fries Shoestring</t>
+          <t>French Fries Crinkle Cut</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Papas Fritas Finas</t>
+          <t>Papas fritas corte ondulado</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Hashbrown 2/10lb.</t>
+          <t>French Fries Homestyle</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Papas Ralladas (Hashbrown) 2/10lb.</t>
+          <t>Papas fritas estilo casero</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Pasta Tortellini</t>
+          <t>French Fries Shoestring</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Pasta Tortellini</t>
+          <t>Papas fritas tipo shoestring</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pizza Crust Cauliflower</t>
+          <t>Hashbrown 2/10lb.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Masa de Pizza de Coliflor</t>
+          <t>Hashbrown 2/10 lb.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Tater Tots</t>
+          <t>Pasta Tortellini</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Croquetas de Papa (Tater Tots)</t>
+          <t>Pasta tortellini</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Tiramisu (ea.)</t>
+          <t>Pizza Crust Cauliflower</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Tiramisú (c/u)</t>
+          <t>Base de pizza de coliflor</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>French Fries 3/8th" Straight</t>
+          <t>Tater Tots</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Papas Fritas Rectas 3/8"</t>
+          <t>Tater tots</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Biscuits 1/24 cs.</t>
+          <t>Tiramisu (ea.)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Panecillos 1/24 caja</t>
+          <t>Tiramisú (unidad)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t> </t>
+          <t>Tortillas Chips uncooked</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t> </t>
+          <t>Totopos sin cocinar</t>
         </is>
       </c>
     </row>
@@ -2631,606 +3252,726 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>l1: English</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>l2: Español</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GROCERY DRY</t>
+          <t>@category: Dry Grocery</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GROCERY DRY</t>
+          <t>@category: Dry Grocery</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Baguettes</t>
+          <t>Banana Peppers sliced 1gal.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Baguettes</t>
+          <t>Chiles banana rebanados 1 gal.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Basalmic Glaze</t>
+          <t>Barbecue Sauce 1 gal.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Glaseado Balsámico</t>
+          <t>Salsa barbecue 1 gal.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Bread Crumbs Panko 25lb.</t>
+          <t>Basalmic Glaze</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Pan Rallado Panko 25lb.</t>
+          <t>Glaseado balsámico</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bread Sliced Sandwich</t>
+          <t>Black Olives Sliced #10 can/cs.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pan de Molde en Rebanadas</t>
+          <t>Aceitunas negras rebanadas lata #10/caja</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Buns Hamburger</t>
+          <t>Bread Baguettes</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Pan para Hamburguesas</t>
+          <t>Baguettes</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Buns Hot Dog</t>
+          <t>Bread Brioche Buns</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Pan para Hot Dogs</t>
+          <t>Pan brioche para hamburguesa</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Croutons 4/2.5lbs.</t>
+          <t>Bread Crumbs Panko 25lb.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Crutones 4/2.5lbs.</t>
+          <t>Pan molido panko 25 lb.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dressing Caesar 1 gal</t>
+          <t>Bread Hawaiian</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Aderezo César 1 galón</t>
+          <t>Pan hawaiano</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dressing Italian 1 gal.</t>
+          <t>Bread Sliced Sandwich</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Aderezo Italiano 1 galón</t>
+          <t>Pan de sándwich rebanado</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dressing Mix Italian packet</t>
+          <t>Brown Sugar 1lb.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mezcla de Aderezo Italiano en paquete</t>
+          <t>Azúcar morena 1 lb.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dressing Mix Ranch packet</t>
+          <t>Buns Hamburger</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Mezcla de Aderezo Ranchero en paquete</t>
+          <t>Pan para hamburguesa</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Dressing Vinagrette 1 gal.</t>
+          <t>Buns Hot Dog</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Vinagreta 1 galón</t>
+          <t>Pan para hot dog</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Flour High Gluten All Trump 25lb.</t>
+          <t>Chocolate for Cannoli #10 can</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Harina de Alto Gluten All Trump 25lb.</t>
+          <t>Chocolate para cannoli lata #10</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Flour High Gluten All Trump 50lb.</t>
+          <t>Cole Slaw Dressing 1gal.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Harina de Alto Gluten All Trump 50lb.</t>
+          <t>Aderezo para cole slaw 1 gal.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Tortillas Flour 10"</t>
+          <t>Cole Slaw mix bag</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tortillas de Harina 10"</t>
+          <t>Bolsa de mezcla para cole slaw</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Fry Oil</t>
+          <t>Croutons 4/2.5lbs.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Aceite para Freír</t>
+          <t>Crutones 4/2.5 lb.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Garlic Minced in water</t>
+          <t>Dressing Caesar 1 gal</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Ajo Picado en agua</t>
+          <t>Aderezo César 1 gal.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Garlic Powder 5lb.</t>
+          <t>Dressing Italian 1 gal.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Ajo en Polvo 5lb.</t>
+          <t>Aderezo italiano 1 gal.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Hot Sauce Red Hot 1 gal.</t>
+          <t>Dressing Mix Italian packet</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Salsa Picante Red Hot 1 galón</t>
+          <t>Mezcla para aderezo italiano, sobre</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Jalapeno Sliced #10</t>
+          <t>Dressing Mix Ranch cs.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Jalapeño en Rodajas lata #10</t>
+          <t>Mezcla para aderezo ranch (caja)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Mayonnaise 4/1 gal.</t>
+          <t>Dressing Mix Ranch packet</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mayonesa 4/1 galón</t>
+          <t>Mezcla para aderezo ranch, sobre</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Olive Ripe Sliced #10 </t>
+          <t>Dressing Vinagrette 1 gal.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aceitunas Maduras en Rodajas lata #10 </t>
+          <t>Vinagreta 1 gal.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Onion minced dried</t>
+          <t>Everything Bagel</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Cebolla Picada Seca</t>
+          <t>Bagel everything</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Onion Powder</t>
+          <t>Flour High Gluten All Trump 25lb.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Cebolla en Polvo</t>
+          <t>Harina alta en gluten All Trump 25 lb.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Pan Spray cs</t>
+          <t>Flour High Gluten All Trump 50lb.</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Aerosol para Sartén caja</t>
+          <t>Harina alta en gluten All Trump 50 lb.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Parmesan Packets</t>
+          <t>Fry Oil</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Paquetes de Queso Parmesano</t>
+          <t>Aceite para freír</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Parsley minced dried</t>
+          <t>Garlic Minced in water</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Perejil Picado Seco</t>
+          <t>Ajo picado en agua</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Pasta Fettucine 10"</t>
+          <t>Garlic Powder 5lb.</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Pasta Fettuccine 10"</t>
+          <t>Ajo en polvo 5 lb.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Pasta Lasagna 10"</t>
+          <t>Hot Sauce Red Hot 1 gal.</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Pasta Lasaña 10"</t>
+          <t>Salsa picante Red Hot 1 gal.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Pasta Penne Rigate</t>
+          <t>Jalapeno Sliced #10</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Pasta Penne Rigate</t>
+          <t>Jalapeño rebanado #10</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Pasta Rotini Tri Color</t>
+          <t>Mayonnaise 4/1 gal.</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Pasta Rotini Tricolor</t>
+          <t>Mayonesa 4/1 gal.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Pasta Spaghetti 10"</t>
+          <t>Olive Ripe Sliced #10</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Pasta Espagueti 10"</t>
+          <t>Aceituna madura rebanada #10</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Pepperoncini Whole 1 gal.</t>
+          <t>Onion minced dried</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Pepperoncini Entero 1 galón</t>
+          <t>Cebolla seca picada</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Pineapple tidbits #10</t>
+          <t>Onion Powder</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Trozos de Piña lata #10</t>
+          <t>Cebolla en polvo</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Ranch Dressing mix cs.</t>
+          <t>Oreos pkg.</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Mezcla para Aderezo Ranchero caja</t>
+          <t>Galletas Oreo, paquete</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Red Pepper Packets</t>
+          <t>Packets Parmesan</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Paquetes de Chile Rojo</t>
+          <t>Sobres de parmesano</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Salsa Fire Roasted #10</t>
+          <t>Packets Red Pepper cs.</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Salsa Asada al Fuego lata #10</t>
+          <t>Sobres de chile rojo (caja)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Salt 50lb.</t>
+          <t>Pan Spray cs</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Sal 50lb.</t>
+          <t>Spray para sartén (caja)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Sugar 50lb.</t>
+          <t>Parsley minced dried</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Azúcar 50lb.</t>
+          <t>Perejil seco picado</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Tomato Paste cs.</t>
+          <t>Pasta Fettucine 10"</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Pasta de Tomate caja</t>
+          <t>Pasta fettuccine 10"</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Tomato Sauce cs.</t>
+          <t>Pasta Lasagna 10"</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Salsa de Tomate caja</t>
+          <t>Pasta para lasaña 10"</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Vinegar Red 1 gal</t>
+          <t>Pasta Penne Rigate</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Vinagre Tinto 1 galón</t>
+          <t>Pasta penne rigate</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Vinegar White 1 gal</t>
+          <t>Pasta Rotini Tri Color</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Vinagre Blanco 1 galón</t>
+          <t>Pasta rotini tricolor</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yeast </t>
+          <t>Pasta Spaghetti 10"</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Levadura</t>
+          <t>Pasta espagueti 10"</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Chocolate for Cannoli #10 can</t>
+          <t>Pepperoncini Whole 1 gal.</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Chocolate para Cannoli lata #10</t>
+          <t>Pepperoncini entero 1 gal.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Texas Toast</t>
+          <t>Pineapple tidbits #10</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Tostada Texana</t>
+          <t>Piña en trozos #10</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Everything Bagel</t>
+          <t>Plain Bagel</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Bagel Todo (Everything)</t>
+          <t>Bagel natural</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Plain Bagel</t>
+          <t>Salsa Fire Roasted #10</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Bagel Sencillo</t>
+          <t>Salsa fire roasted #10</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Salt 50lb.</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Sal 50 lb.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Sugar 50lb.</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Azúcar 50 lb.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Sugar Powdered bag</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Azúcar glass, bolsa</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Texas Toast</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Texas toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Tomato Paste cs.</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Pasta de tomate (caja)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Tomato Sauce cs.</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Salsa de tomate (caja)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Tortillas Flour 10"</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Tortillas de harina 10"</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Vinegar Red 1 gal</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Vinagre rojo 1 gal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Vinegar White 1 gal</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Vinagre blanco 1 gal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Yeast</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Levadura</t>
         </is>
       </c>
     </row>
@@ -3251,240 +3992,240 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>l1: English</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>l2: Español</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MEATS</t>
+          <t>@category: Meats</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Carnes</t>
+          <t>@category: Carnes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bacon Sliced 1cs</t>
+          <t>Bacon Bits (case)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tocino en Rebanadas 1 caja</t>
+          <t>Tocino en trocitos (caja)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Canadian Bacon</t>
+          <t>Bacon Sliced 1cs</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tocino Canadiense</t>
+          <t>Tocino rebanado 1 caja</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ground Beef 73/27 lbs</t>
+          <t>Brisket (each)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Carne Molida 73/27 lbs</t>
+          <t>Brisket (unidad)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ground Beef 80/20 lbs</t>
+          <t>Canadian Bacon (case)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Carne Molida 80/20 lbs</t>
+          <t>Tocino canadiense (caja)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ground Beef 90/10 lbs</t>
+          <t>Catfish/Swai cs.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Carne Molida 90/10 lbs</t>
+          <t>Bagre/Swai (caja)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Italian Sausage Rope</t>
+          <t>Chicken Breast (case)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Salchicha Italiana en Cuerda</t>
+          <t>Pechuga de pollo (caja)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pepperoni</t>
+          <t>Chicken Wings (case)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pepperoni</t>
+          <t>Alitas de pollo (caja)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Philly Meat</t>
+          <t>Ground Beef 73/27 lbs</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Carne para Philly</t>
+          <t>Carne molida 73/27 lb.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Chicken Breast</t>
+          <t>Ground Beef 80/20 lbs</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Pechuga de Pollo</t>
+          <t>Carne molida 80/20 lb.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Chicken Wings</t>
+          <t>Ground Beef 90/10 lbs</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Alitas de Pollo</t>
+          <t>Carne molida 90/10 lb.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bacon Bits </t>
+          <t>Hot Dogs (each)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trozos de Tocino </t>
+          <t>Hot dogs (unidad)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Shrimp 21-25 raw peeled 5/2lb.</t>
+          <t>Hot Links (each)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Camarones 21-25 crudos y pelados 5/2lb.</t>
+          <t>Salchichas hot links (unidad)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Brisket</t>
+          <t>Italian Sausage Rope (case)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Pecho de Res (Brisket)</t>
+          <t>Salchicha italiana en tira (caja)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Pork Butt</t>
+          <t>Pepperoni (case)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Paleta de Cerdo</t>
+          <t>Pepperoni (caja)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Polish Sausage</t>
+          <t>Philly Meat (case)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Salchicha Polaca</t>
+          <t>Carne tipo Philly (caja)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Hot Links</t>
+          <t>Polish Sausage (each)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Salchichas Picantes</t>
+          <t>Salchicha polaca (unidad)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Hot Dogs</t>
+          <t>Pork Butt (each)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Hot Dogs</t>
+          <t>Pork butt (unidad)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Catfish/Swai cs.</t>
+          <t>Shrimp 21-25 raw peeled 5/2lb. (case)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bagre/Swai caja</t>
+          <t>Camarón 21-25 crudo pelado 5/2 lb. (caja)</t>
         </is>
       </c>
     </row>

</xml_diff>